<commit_message>
First version of BTRG is ready
</commit_message>
<xml_diff>
--- a/Additional/Tests.xlsx
+++ b/Additional/Tests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iakob\Desktop\programing\tensornetworks\Additional\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergey\Desktop\programming\tensornetworks\Additional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013CB77A-90D6-4C45-AD6E-255B42C6C69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27A5BF9C-5C5D-4534-99CA-15AC05C698C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4E5A4C81-6162-4430-A263-13FAAFDD787D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="31920" xr2:uid="{4E5A4C81-6162-4430-A263-13FAAFDD787D}"/>
   </bookViews>
   <sheets>
     <sheet name="HOTRG" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>TRG(24)</t>
   </si>
@@ -66,6 +66,18 @@
   </si>
   <si>
     <t>Error (HOTRG24)</t>
+  </si>
+  <si>
+    <t>BTRG(10)</t>
+  </si>
+  <si>
+    <t>BTRG(24)</t>
+  </si>
+  <si>
+    <t>Error(BTRG10)</t>
+  </si>
+  <si>
+    <t>Error(BTRG(24)</t>
   </si>
 </sst>
 </file>
@@ -746,6 +758,303 @@
             </c:ext>
           </c:extLst>
         </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>HOTRG!$N$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Error(BTRG(24)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>HOTRG!$A$2:$A$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>2.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.1199999999999899</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.1299999999999901</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.1399999999999899</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.1499999999999901</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.1599999999999899</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.1699999999999902</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.1799999999999899</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.1899999999999902</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.19999999999999</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.2099999999999902</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.21999999999999</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.2299999999999902</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.23999999999999</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.2499999999999898</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.25999999999999</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.2699999999999898</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.27999999999999</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2.2899999999999898</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2.2999999999999901</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.3099999999999898</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2.3199999999999901</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2.3299999999999899</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2.3399999999999901</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2.3499999999999899</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2.3599999999999901</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2.3699999999999899</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2.3799999999999901</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2.3899999999999899</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2.3999999999999901</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>2.4099999999999899</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>2.4199999999999902</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>2.4299999999999899</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>2.4399999999999902</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>2.44999999999999</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>2.4599999999999902</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>2.46999999999999</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2.4799999999999902</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2.48999999999999</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>2.4999999999999898</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>HOTRG!$N$2:$N$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>1.4282341975757618E-9</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.6848838990668469E-9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.9982934196249857E-9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.340741156459103E-9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.6714543910344446E-9</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.1494280516852768E-9</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.7515747175476122E-9</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.518220020344188E-9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.4328079812648866E-9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>6.6009695487423414E-9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>7.8077725396141773E-9</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>9.7309275082224644E-9</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.2169469432166125E-8</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.5631689942452454E-8</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.9760985736638759E-8</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.6671470587658064E-8</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3.9238729265811401E-8</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5.4000796834152709E-8</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3.3903976182081408E-8</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2.4802297993176126E-8</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.9178904353545079E-8</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1.5486933069297493E-8</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1.2560437689934645E-8</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1.0406611017366174E-8</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>8.5489925139015099E-9</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>7.3821631030313029E-9</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>6.2955358703931097E-9</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>5.4055120379814525E-9</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>4.6616626114825976E-9</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>4.0526991762490638E-9</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>3.5451996893698379E-9</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>3.1156057733738862E-9</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>2.7536249946891189E-9</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>2.4487831762343149E-9</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>2.1890194101814586E-9</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>1.9443374688066228E-9</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>1.7501962101817981E-9</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>1.5637844352767161E-9</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>1.4160669303819873E-9</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>1.2871084198451399E-9</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>1.1716425607488645E-9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-75A7-4756-8E35-ED3071E39C6F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -1081,7 +1390,7 @@
                 <c:order val="1"/>
                 <c:tx>
                   <c:strRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>HOTRG!$H$1</c15:sqref>
@@ -1110,7 +1419,7 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>HOTRG!$A$2:$A$42</c15:sqref>
@@ -1248,7 +1557,7 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>HOTRG!$H$2:$H$42</c15:sqref>
@@ -1385,7 +1694,7 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000001-ACD7-433B-AAFB-3E5A97ED6BF9}"/>
                   </c:ext>
@@ -1465,7 +1774,7 @@
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
           <c:max val="5.0000000000000021E-6"/>
-          <c:min val="5.0000000000000029E-12"/>
+          <c:min val="4.0000000000000022E-10"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1538,10 +1847,10 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.28708989501312338"/>
-          <c:y val="0.92287497822958398"/>
-          <c:w val="0.4645797091497284"/>
-          <c:h val="6.5483578231417233E-2"/>
+          <c:x val="0.13391704045747016"/>
+          <c:y val="0.92287511547090118"/>
+          <c:w val="0.69710524697617404"/>
+          <c:h val="6.2849601900321128E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -1617,7 +1926,1181 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="ru-RU"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>HOTRG!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Error (TRG10)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>HOTRG!$A$2:$A$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>2.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.1199999999999899</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.1299999999999901</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.1399999999999899</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.1499999999999901</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.1599999999999899</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.1699999999999902</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.1799999999999899</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.1899999999999902</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.19999999999999</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.2099999999999902</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.21999999999999</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.2299999999999902</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.23999999999999</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.2499999999999898</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.25999999999999</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.2699999999999898</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.27999999999999</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2.2899999999999898</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2.2999999999999901</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.3099999999999898</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2.3199999999999901</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2.3299999999999899</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2.3399999999999901</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2.3499999999999899</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2.3599999999999901</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2.3699999999999899</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2.3799999999999901</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2.3899999999999899</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2.3999999999999901</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>2.4099999999999899</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>2.4199999999999902</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>2.4299999999999899</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>2.4399999999999902</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>2.44999999999999</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>2.4599999999999902</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>2.46999999999999</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2.4799999999999902</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2.48999999999999</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>2.4999999999999898</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>HOTRG!$D$2:$D$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>5.1255469878386251E-6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5.5808663191880825E-6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.076785450170874E-6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6.6168690703305444E-6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7.2049109748340001E-6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7.8448906360994997E-6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8.5408849496149131E-6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9.2969045091262359E-6</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0116599588272379E-5</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.1002733285581101E-5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1956222570330688E-5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.2974342484484147E-5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.4047198323430266E-5</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.5150265720187406E-5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.6226772467153872E-5</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.7137858538185391E-5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.7462189497718938E-5</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.4076735193713219E-5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.1529645519314791E-5</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.0330172572792229E-5</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>9.5604489396272641E-6</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>9.0189965776810155E-6</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>8.588626002503652E-6</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>8.2579161145845958E-6</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>7.9600973104110295E-6</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>7.7309974632067124E-6</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>7.4963739555844455E-6</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>7.3238388386132058E-6</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>7.169815815277758E-6</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>7.0306201818137737E-6</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>6.9034626550834588E-6</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>6.7516846173898415E-6</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>6.6444440969259944E-6</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>6.5449949839813115E-6</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>6.4522285291301884E-6</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>6.3652202786368406E-6</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>6.2831811622476863E-6</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>6.2054222514928981E-6</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>6.0956233050024622E-6</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>6.0232755140221528E-6</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>5.9544812879286368E-6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2676-4216-9047-F73D3DCD5D8D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>HOTRG!$H$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Error (HOTRG10)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>HOTRG!$A$2:$A$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>2.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.1199999999999899</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.1299999999999901</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.1399999999999899</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.1499999999999901</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.1599999999999899</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.1699999999999902</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.1799999999999899</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.1899999999999902</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.19999999999999</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.2099999999999902</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.21999999999999</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.2299999999999902</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.23999999999999</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.2499999999999898</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.25999999999999</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.2699999999999898</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.27999999999999</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2.2899999999999898</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2.2999999999999901</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.3099999999999898</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2.3199999999999901</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2.3299999999999899</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2.3399999999999901</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2.3499999999999899</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2.3599999999999901</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2.3699999999999899</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2.3799999999999901</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2.3899999999999899</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2.3999999999999901</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>2.4099999999999899</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>2.4199999999999902</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>2.4299999999999899</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>2.4399999999999902</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>2.44999999999999</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>2.4599999999999902</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>2.46999999999999</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2.4799999999999902</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2.48999999999999</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>2.4999999999999898</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>HOTRG!$H$2:$H$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>7.6956423900043092E-8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.1185741188857179E-7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.5174722012289976E-7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.974628045520177E-7</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.5002409997920694E-7</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.1066545247426802E-7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.8087006559717196E-7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.6241798157264924E-7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.5747542793138649E-7</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>6.6876388093994876E-7</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>7.9985858947306809E-7</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>9.5563719393343405E-7</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.1428129269575038E-6</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.370454023152945E-6</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.651065626773196E-6</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.0038032094715774E-6</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.4576908053131064E-6</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.9731299696633684E-6</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.8432345584583629E-6</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2.618688157762783E-6</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2.4056400874661321E-6</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.1620653846143867E-6</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1.993660867505298E-6</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1.8345409502629195E-6</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1.6491654378780751E-6</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1.4415791667055089E-6</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1.3197866729486307E-6</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1.2094394108430606E-6</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1.1079639669064889E-6</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1.0139121854324529E-6</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>9.2652983540997269E-7</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>8.4540742673056002E-7</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>7.3974419290134819E-7</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>6.7163882000453867E-7</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>6.0914128841016435E-7</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>5.5109409380360574E-7</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>4.7194561758612252E-7</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>4.2255046706074495E-7</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>3.7792103479983297E-7</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2.2969375357284605E-7</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>1.9798409245375126E-7</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-2676-4216-9047-F73D3DCD5D8D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>HOTRG!$M$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Error(BTRG10)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>HOTRG!$A$2:$A$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>2.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.1199999999999899</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.1299999999999901</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.1399999999999899</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.1499999999999901</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.1599999999999899</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.1699999999999902</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.1799999999999899</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.1899999999999902</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.19999999999999</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.2099999999999902</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.21999999999999</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.2299999999999902</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.23999999999999</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.2499999999999898</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.25999999999999</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.2699999999999898</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.27999999999999</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2.2899999999999898</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2.2999999999999901</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.3099999999999898</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2.3199999999999901</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2.3299999999999899</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2.3399999999999901</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2.3499999999999899</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2.3599999999999901</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2.3699999999999899</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2.3799999999999901</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2.3899999999999899</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2.3999999999999901</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>2.4099999999999899</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>2.4199999999999902</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>2.4299999999999899</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>2.4399999999999902</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>2.44999999999999</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>2.4599999999999902</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>2.46999999999999</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2.4799999999999902</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2.48999999999999</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>2.4999999999999898</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>HOTRG!$M$2:$M$42</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="41"/>
+                <c:pt idx="0">
+                  <c:v>2.3101496182675874E-7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.5442201079250992E-7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.8081165726057122E-7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.1069002437433824E-7</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.4467527809667331E-7</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.8352838549471358E-7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.2819342371824831E-7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.7985351825374778E-7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.4001290050731399E-7</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>6.1061695522113268E-7</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>6.9422698301124797E-7</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>7.9429310184675472E-7</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>9.1561649051552507E-7</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.0651636422887023E-6</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.253690325553336E-6</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.499584192377057E-6</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.8414590247095575E-6</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.4865904605375633E-6</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.6222459942326637E-6</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2.5023433061210909E-6</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2.3386490682897332E-6</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.1560482194038499E-6</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2.009036657146801E-6</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1.8292392216512354E-6</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1.6987122543055122E-6</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1.5372538234581512E-6</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1.4247068866879431E-6</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1.3223173590537485E-6</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1.2285209924911555E-6</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1.1096750424099966E-6</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>1.0290537066914851E-6</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>9.5601265526212842E-7</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>8.8948324483695274E-7</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>8.2859470862395312E-7</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>7.7259858233258427E-7</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>7.0494654269559476E-7</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>6.5531154513909229E-7</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>6.1023181541219884E-7</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>5.6915196677831403E-7</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>5.315964631824599E-7</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>4.9715971661701275E-7</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-2676-4216-9047-F73D3DCD5D8D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1745793280"/>
+        <c:axId val="1745793760"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1745793280"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="2.5"/>
+          <c:min val="2.1"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1745793760"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1745793760"/>
+        <c:scaling>
+          <c:logBase val="10"/>
+          <c:orientation val="minMax"/>
+          <c:max val="5.0000000000000023E-5"/>
+          <c:min val="4.0000000000000021E-8"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1745793280"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="ru-RU"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="ru-RU"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -2173,20 +3656,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>175260</xdr:colOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>264557</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:rowOff>135017</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>541020</xdr:colOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>23099</xdr:colOff>
       <xdr:row>18</xdr:row>
-      <xdr:rowOff>121920</xdr:rowOff>
+      <xdr:rowOff>115967</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2211,13 +4210,49 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>258960</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>60125</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>166688</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>172640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Диаграмма 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5263B89B-E757-7D39-48AE-3F571ADE76B5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office 2013–2022">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2255,7 +4290,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2361,7 +4396,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2503,7 +4538,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2511,19 +4546,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7195F39-8342-4B20-915A-AACA967BE21D}">
-  <dimension ref="A1:O42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AA42"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="12.88671875" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.21875" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" customWidth="1"/>
-    <col min="9" max="9" width="10.44140625" customWidth="1"/>
-    <col min="10" max="10" width="14.5546875" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.140625" customWidth="1"/>
+    <col min="9" max="9" width="10.42578125" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" customWidth="1"/>
+    <col min="14" max="14" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -2554,8 +4591,20 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2.1</v>
       </c>
@@ -2566,7 +4615,7 @@
         <v>2.0688308534154101</v>
       </c>
       <c r="D2">
-        <f>1-C2/B2</f>
+        <f t="shared" ref="D2:D42" si="0">1-C2/B2</f>
         <v>5.1255469878386251E-6</v>
       </c>
       <c r="E2">
@@ -2580,7 +4629,7 @@
         <v>2.06884129814887</v>
       </c>
       <c r="H2">
-        <f>ABS(1-G2/B2)</f>
+        <f t="shared" ref="H2:H42" si="1">ABS(1-G2/B2)</f>
         <v>7.6956423900043092E-8</v>
       </c>
       <c r="I2">
@@ -2590,8 +4639,31 @@
         <f>ABS(1-I2/B2)</f>
         <v>1.9735567402534571E-8</v>
       </c>
+      <c r="K2">
+        <v>2.0688409794261799</v>
+      </c>
+      <c r="L2">
+        <v>2.06884145440472</v>
+      </c>
+      <c r="M2">
+        <f>ABS(1-K2/B2)</f>
+        <v>2.3101496182675874E-7</v>
+      </c>
+      <c r="N2">
+        <f>ABS(1-L2/B2)</f>
+        <v>1.4282341975757618E-9</v>
+      </c>
+      <c r="Y2">
+        <v>2.1</v>
+      </c>
+      <c r="Z2">
+        <v>2.06884145440472</v>
+      </c>
+      <c r="AA2">
+        <v>10.822773599997101</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2.11</v>
       </c>
@@ -2602,32 +4674,55 @@
         <v>2.07078997628544</v>
       </c>
       <c r="D3">
-        <f>1-C3/B3</f>
+        <f t="shared" si="0"/>
         <v>5.5808663191880825E-6</v>
       </c>
       <c r="E3">
         <v>2.0708010313785401</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F42" si="0">1-E3/B3</f>
+        <f t="shared" ref="F3:F42" si="2">1-E3/B3</f>
         <v>2.4230879780429149E-7</v>
       </c>
       <c r="G3">
         <v>2.07080130151747</v>
       </c>
       <c r="H3">
-        <f>ABS(1-G3/B3)</f>
+        <f t="shared" si="1"/>
         <v>1.1185741188857179E-7</v>
       </c>
       <c r="I3">
         <v>2.0708014900949601</v>
       </c>
       <c r="J3">
-        <f t="shared" ref="J3:J42" si="1">ABS(1-I3/B3)</f>
+        <f t="shared" ref="J3:J42" si="3">ABS(1-I3/B3)</f>
         <v>2.0792436772332223E-8</v>
       </c>
+      <c r="K3">
+        <v>2.0708010062944799</v>
+      </c>
+      <c r="L3">
+        <v>2.0708015296629099</v>
+      </c>
+      <c r="M3">
+        <f t="shared" ref="M3:M42" si="4">ABS(1-K3/B3)</f>
+        <v>2.5442201079250992E-7</v>
+      </c>
+      <c r="N3">
+        <f t="shared" ref="N3:N42" si="5">ABS(1-L3/B3)</f>
+        <v>1.6848838990668469E-9</v>
+      </c>
+      <c r="Y3">
+        <v>2.11</v>
+      </c>
+      <c r="Z3">
+        <v>2.0708015296629099</v>
+      </c>
+      <c r="AA3">
+        <v>22.873911099973999</v>
+      </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2.1199999999999899</v>
       </c>
@@ -2638,32 +4733,55 @@
         <v>2.07279611732646</v>
       </c>
       <c r="D4">
-        <f>1-C4/B4</f>
+        <f t="shared" si="0"/>
         <v>6.076785450170874E-6</v>
       </c>
       <c r="E4">
         <v>2.07280814885761</v>
       </c>
       <c r="F4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.7232743504690404E-7</v>
       </c>
       <c r="G4">
         <v>2.07280839879733</v>
       </c>
       <c r="H4">
-        <f>ABS(1-G4/B4)</f>
+        <f t="shared" si="1"/>
         <v>1.5174722012289976E-7</v>
       </c>
       <c r="I4">
         <v>2.0728086648996298</v>
       </c>
       <c r="J4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.3369575830045619E-8</v>
       </c>
+      <c r="K4">
+        <v>2.0728081312714401</v>
+      </c>
+      <c r="L4">
+        <v>2.0728087091982101</v>
+      </c>
+      <c r="M4">
+        <f t="shared" si="4"/>
+        <v>2.8081165726057122E-7</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="5"/>
+        <v>1.9982934196249857E-9</v>
+      </c>
+      <c r="Y4">
+        <v>2.1199999999999899</v>
+      </c>
+      <c r="Z4">
+        <v>2.0728087091982101</v>
+      </c>
+      <c r="AA4">
+        <v>34.9319418000523</v>
+      </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2.1299999999999901</v>
       </c>
@@ -2674,32 +4792,55 @@
         <v>2.07485060388731</v>
       </c>
       <c r="D5">
-        <f>1-C5/B5</f>
+        <f t="shared" si="0"/>
         <v>6.6168690703305444E-6</v>
       </c>
       <c r="E5">
         <v>2.0748637134083201</v>
       </c>
       <c r="F5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.9861452155444113E-7</v>
       </c>
       <c r="G5">
         <v>2.0748639232844099</v>
       </c>
       <c r="H5">
-        <f>ABS(1-G5/B5)</f>
+        <f t="shared" si="1"/>
         <v>1.974628045520177E-7</v>
       </c>
       <c r="I5">
         <v>2.0748642817179901</v>
       </c>
       <c r="J5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.4712435098273033E-8</v>
       </c>
+      <c r="K5">
+        <v>2.07486368835329</v>
+      </c>
+      <c r="L5">
+        <v>2.0748643281362198</v>
+      </c>
+      <c r="M5">
+        <f t="shared" si="4"/>
+        <v>3.1069002437433824E-7</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="5"/>
+        <v>2.340741156459103E-9</v>
+      </c>
+      <c r="Y5">
+        <v>2.1299999999999901</v>
+      </c>
+      <c r="Z5">
+        <v>2.0748643281362198</v>
+      </c>
+      <c r="AA5">
+        <v>46.990211399970498</v>
+      </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2.1399999999999899</v>
       </c>
@@ -2710,32 +4851,55 @@
         <v>2.0769548555288702</v>
       </c>
       <c r="D6">
-        <f>1-C6/B6</f>
+        <f t="shared" si="0"/>
         <v>7.2049109748340001E-6</v>
       </c>
       <c r="E6">
         <v>2.0769691391204601</v>
       </c>
       <c r="F6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>3.2778091108021101E-7</v>
       </c>
       <c r="G6">
         <v>2.0769693006190102</v>
       </c>
       <c r="H6">
-        <f>ABS(1-G6/B6)</f>
+        <f t="shared" si="1"/>
         <v>2.5002409997920694E-7</v>
       </c>
       <c r="I6">
         <v>2.07696976559411</v>
       </c>
       <c r="J6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.6152238485899204E-8</v>
       </c>
+      <c r="K6">
+        <v>2.0769691040313698</v>
+      </c>
+      <c r="L6">
+        <v>2.07696981436299</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="4"/>
+        <v>3.4467527809667331E-7</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="5"/>
+        <v>2.6714543910344446E-9</v>
+      </c>
+      <c r="Y6">
+        <v>2.1399999999999899</v>
+      </c>
+      <c r="Z6">
+        <v>2.07696981436299</v>
+      </c>
+      <c r="AA6">
+        <v>59.067980400053699</v>
+      </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2.1499999999999901</v>
       </c>
@@ -2746,32 +4910,55 @@
         <v>2.0791103983664501</v>
       </c>
       <c r="D7">
-        <f>1-C7/B7</f>
+        <f t="shared" si="0"/>
         <v>7.8448906360994997E-6</v>
       </c>
       <c r="E7">
         <v>2.0791259601658001</v>
       </c>
       <c r="F7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>3.6011383841572098E-7</v>
       </c>
       <c r="G7">
         <v>2.0791260629752601</v>
       </c>
       <c r="H7">
-        <f>ABS(1-G7/B7)</f>
+        <f t="shared" si="1"/>
         <v>3.1066545247426802E-7</v>
       </c>
       <c r="I7">
         <v>2.0791266512743598</v>
       </c>
       <c r="J7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.7710547745307679E-8</v>
       </c>
+      <c r="K7">
+        <v>2.07912591148399</v>
+      </c>
+      <c r="L7">
+        <v>2.0791267023400399</v>
+      </c>
+      <c r="M7">
+        <f t="shared" si="4"/>
+        <v>3.8352838549471358E-7</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="5"/>
+        <v>3.1494280516852768E-9</v>
+      </c>
+      <c r="Y7">
+        <v>2.1499999999999901</v>
+      </c>
+      <c r="Z7">
+        <v>2.0791267023400399</v>
+      </c>
+      <c r="AA7">
+        <v>71.139418700011404</v>
+      </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2.1599999999999899</v>
       </c>
@@ -2782,32 +4969,55 @@
         <v>2.0813188830070701</v>
       </c>
       <c r="D8">
-        <f>1-C8/B8</f>
+        <f t="shared" si="0"/>
         <v>8.5408849496149131E-6</v>
       </c>
       <c r="E8">
         <v>2.0813358354970402</v>
       </c>
       <c r="F8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>3.9588356659514545E-7</v>
       </c>
       <c r="G8">
         <v>2.08133586674519</v>
       </c>
       <c r="H8">
-        <f>ABS(1-G8/B8)</f>
+        <f t="shared" si="1"/>
         <v>3.8087006559717196E-7</v>
       </c>
       <c r="I8">
         <v>2.0813365982390302</v>
       </c>
       <c r="J8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.9416187707909103E-8</v>
       </c>
+      <c r="K8">
+        <v>2.0813357682493501</v>
+      </c>
+      <c r="L8">
+        <v>2.0813366516557301</v>
+      </c>
+      <c r="M8">
+        <f t="shared" si="4"/>
+        <v>4.2819342371824831E-7</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="5"/>
+        <v>3.7515747175476122E-9</v>
+      </c>
+      <c r="Y8">
+        <v>2.1599999999999899</v>
+      </c>
+      <c r="Z8">
+        <v>2.0813366516557301</v>
+      </c>
+      <c r="AA8">
+        <v>83.186399300117003</v>
+      </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2.1699999999999902</v>
       </c>
@@ -2818,32 +5028,55 @@
         <v>2.08358210739001</v>
       </c>
       <c r="D9">
-        <f>1-C9/B9</f>
+        <f t="shared" si="0"/>
         <v>9.2969045091262359E-6</v>
       </c>
       <c r="E9">
         <v>2.0836005439582701</v>
       </c>
       <c r="F9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>4.4849062053042843E-7</v>
       </c>
       <c r="G9">
         <v>2.0836005149391998</v>
       </c>
       <c r="H9">
-        <f>ABS(1-G9/B9)</f>
+        <f t="shared" si="1"/>
         <v>4.6241798157264924E-7</v>
       </c>
       <c r="I9">
         <v>2.08360142859717</v>
       </c>
       <c r="J9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.3918594993510567E-8</v>
       </c>
+      <c r="K9">
+        <v>2.08360047861049</v>
+      </c>
+      <c r="L9">
+        <v>2.0836014690198201</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="4"/>
+        <v>4.7985351825374778E-7</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="5"/>
+        <v>4.518220020344188E-9</v>
+      </c>
+      <c r="Y9">
+        <v>2.1699999999999902</v>
+      </c>
+      <c r="Z9">
+        <v>2.0836014690198201</v>
+      </c>
+      <c r="AA9">
+        <v>95.245498999953199</v>
+      </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2.1799999999999899</v>
       </c>
@@ -2854,32 +5087,55 @@
         <v>2.0859020464958</v>
       </c>
       <c r="D10">
-        <f>1-C10/B10</f>
+        <f t="shared" si="0"/>
         <v>1.0116599588272379E-5</v>
       </c>
       <c r="E10">
         <v>2.0859221110895501</v>
       </c>
       <c r="F10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>4.9755213671343057E-7</v>
       </c>
       <c r="G10">
         <v>2.0859219860941698</v>
       </c>
       <c r="H10">
-        <f>ABS(1-G10/B10)</f>
+        <f t="shared" si="1"/>
         <v>5.5747542793138649E-7</v>
       </c>
       <c r="I10">
         <v>2.0859230952146799</v>
       </c>
       <c r="J10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.5758566390976512E-8</v>
       </c>
+      <c r="K10">
+        <v>2.08592202251966</v>
+      </c>
+      <c r="L10">
+        <v>2.0859231376126499</v>
+      </c>
+      <c r="M10">
+        <f t="shared" si="4"/>
+        <v>5.4001290050731399E-7</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="5"/>
+        <v>5.4328079812648866E-9</v>
+      </c>
+      <c r="Y10">
+        <v>2.1799999999999899</v>
+      </c>
+      <c r="Z10">
+        <v>2.0859231376126499</v>
+      </c>
+      <c r="AA10">
+        <v>107.29150560009199</v>
+      </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2.1899999999999902</v>
       </c>
@@ -2890,32 +5146,55 @@
         <v>2.0882808919885698</v>
       </c>
       <c r="D11">
-        <f>1-C11/B11</f>
+        <f t="shared" si="0"/>
         <v>1.1002733285581101E-5</v>
       </c>
       <c r="E11">
         <v>2.0883027149685098</v>
       </c>
       <c r="F11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>5.5263535514438189E-7</v>
       </c>
       <c r="G11">
         <v>2.08830247245686</v>
       </c>
       <c r="H11">
-        <f>ABS(1-G11/B11)</f>
+        <f t="shared" si="1"/>
         <v>6.6876388093994876E-7</v>
       </c>
       <c r="I11">
         <v>2.0883038106174401</v>
       </c>
       <c r="J11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.7975631700094539E-8</v>
       </c>
+      <c r="K11">
+        <v>2.0883025938853099</v>
+      </c>
+      <c r="L11">
+        <v>2.0883038552542299</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="4"/>
+        <v>6.1061695522113268E-7</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="5"/>
+        <v>6.6009695487423414E-9</v>
+      </c>
+      <c r="Y11">
+        <v>2.1899999999999902</v>
+      </c>
+      <c r="Z11">
+        <v>2.0883038552542299</v>
+      </c>
+      <c r="AA11">
+        <v>119.347242100164</v>
+      </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2.19999999999999</v>
       </c>
@@ -2926,32 +5205,55 @@
         <v>2.0907211067875</v>
       </c>
       <c r="D12">
-        <f>1-C12/B12</f>
+        <f t="shared" si="0"/>
         <v>1.1956222570330688E-5</v>
       </c>
       <c r="E12">
         <v>2.0907447964695902</v>
       </c>
       <c r="F12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>6.2549138180045816E-7</v>
       </c>
       <c r="G12">
         <v>2.0907444319120301</v>
       </c>
       <c r="H12">
-        <f>ABS(1-G12/B12)</f>
+        <f t="shared" si="1"/>
         <v>7.9985858947306809E-7</v>
       </c>
       <c r="I12">
         <v>2.0907460401455902</v>
       </c>
       <c r="J12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>3.0643448112321892E-8</v>
       </c>
+      <c r="K12">
+        <v>2.0907446527608999</v>
+      </c>
+      <c r="L12">
+        <v>2.0907460878891899</v>
+      </c>
+      <c r="M12">
+        <f t="shared" si="4"/>
+        <v>6.9422698301124797E-7</v>
+      </c>
+      <c r="N12">
+        <f t="shared" si="5"/>
+        <v>7.8077725396141773E-9</v>
+      </c>
+      <c r="Y12">
+        <v>2.19999999999999</v>
+      </c>
+      <c r="Z12">
+        <v>2.0907460878891899</v>
+      </c>
+      <c r="AA12">
+        <v>131.420531400013</v>
+      </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2.2099999999999902</v>
       </c>
@@ -2962,32 +5264,55 @@
         <v>2.09322550315696</v>
       </c>
       <c r="D13">
-        <f>1-C13/B13</f>
+        <f t="shared" si="0"/>
         <v>1.2974342484484147E-5</v>
       </c>
       <c r="E13">
         <v>2.09325119503987</v>
       </c>
       <c r="F13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>7.0067701651854719E-7</v>
       </c>
       <c r="G13">
         <v>2.0932506613438</v>
       </c>
       <c r="H13">
-        <f>ABS(1-G13/B13)</f>
+        <f t="shared" si="1"/>
         <v>9.5563719393343405E-7</v>
       </c>
       <c r="I13">
         <v>2.0932525887059801</v>
       </c>
       <c r="J13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>3.4887293387519946E-8</v>
       </c>
+      <c r="K13">
+        <v>2.0932509990777501</v>
+      </c>
+      <c r="L13">
+        <v>2.09325264136461</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="4"/>
+        <v>7.9429310184675472E-7</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="5"/>
+        <v>9.7309275082224644E-9</v>
+      </c>
+      <c r="Y13">
+        <v>2.2099999999999902</v>
+      </c>
+      <c r="Z13">
+        <v>2.09325264136461</v>
+      </c>
+      <c r="AA13">
+        <v>143.49993579997599</v>
+      </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2.21999999999999</v>
       </c>
@@ -2998,32 +5323,55 @@
         <v>2.0957973601545299</v>
       </c>
       <c r="D14">
-        <f>1-C14/B14</f>
+        <f t="shared" si="0"/>
         <v>1.4047198323430266E-5</v>
       </c>
       <c r="E14">
         <v>2.09582513723978</v>
       </c>
       <c r="F14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>7.9367697258803105E-7</v>
       </c>
       <c r="G14">
         <v>2.0958244055112898</v>
       </c>
       <c r="H14">
-        <f>ABS(1-G14/B14)</f>
+        <f t="shared" si="1"/>
         <v>1.1428129269575038E-6</v>
       </c>
       <c r="I14">
         <v>2.0958267181144499</v>
       </c>
       <c r="J14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>3.9380544381018012E-8</v>
       </c>
+      <c r="K14">
+        <v>2.0958248816756702</v>
+      </c>
+      <c r="L14">
+        <v>2.0958267751441499</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="4"/>
+        <v>9.1561649051552507E-7</v>
+      </c>
+      <c r="N14">
+        <f t="shared" si="5"/>
+        <v>1.2169469432166125E-8</v>
+      </c>
+      <c r="Y14">
+        <v>2.21999999999999</v>
+      </c>
+      <c r="Z14">
+        <v>2.0958267751441499</v>
+      </c>
+      <c r="AA14">
+        <v>155.588994800113</v>
+      </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2.2299999999999902</v>
       </c>
@@ -3034,32 +5382,55 @@
         <v>2.0984406124381199</v>
       </c>
       <c r="D15">
-        <f>1-C15/B15</f>
+        <f t="shared" si="0"/>
         <v>1.5150265720187406E-5</v>
       </c>
       <c r="E15">
         <v>2.09847051893207</v>
       </c>
       <c r="F15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>8.9871116992767952E-7</v>
       </c>
       <c r="G15">
         <v>2.0984695289927102</v>
       </c>
       <c r="H15">
-        <f>ABS(1-G15/B15)</f>
+        <f t="shared" si="1"/>
         <v>1.370454023152945E-6</v>
       </c>
       <c r="I15">
         <v>2.09847230837318</v>
       </c>
       <c r="J15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>4.5976053741902945E-8</v>
       </c>
+      <c r="K15">
+        <v>2.0984701696361499</v>
+      </c>
+      <c r="L15">
+        <v>2.09847237204999</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="4"/>
+        <v>1.0651636422887023E-6</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="5"/>
+        <v>1.5631689942452454E-8</v>
+      </c>
+      <c r="Y15">
+        <v>2.2299999999999902</v>
+      </c>
+      <c r="Z15">
+        <v>2.09847237204999</v>
+      </c>
+      <c r="AA15">
+        <v>168.195618000114</v>
+      </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2.23999999999999</v>
       </c>
@@ -3070,32 +5441,55 @@
         <v>2.1011601837241201</v>
       </c>
       <c r="D16">
-        <f>1-C16/B16</f>
+        <f t="shared" si="0"/>
         <v>1.6226772467153872E-5</v>
       </c>
       <c r="E16">
         <v>2.10119213885626</v>
       </c>
       <c r="F16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.0186917797083694E-6</v>
       </c>
       <c r="G16">
         <v>2.1011908101159502</v>
       </c>
       <c r="H16">
-        <f>ABS(1-G16/B16)</f>
+        <f t="shared" si="1"/>
         <v>1.651065626773196E-6</v>
       </c>
       <c r="I16">
         <v>2.1011941658709601</v>
       </c>
       <c r="J16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>5.3995311666277246E-8</v>
       </c>
+      <c r="K16">
+        <v>2.1011916450786599</v>
+      </c>
+      <c r="L16">
+        <v>2.1011942378039299</v>
+      </c>
+      <c r="M16">
+        <f t="shared" si="4"/>
+        <v>1.253690325553336E-6</v>
+      </c>
+      <c r="N16">
+        <f t="shared" si="5"/>
+        <v>1.9760985736638759E-8</v>
+      </c>
+      <c r="Y16">
+        <v>2.23999999999999</v>
+      </c>
+      <c r="Z16">
+        <v>2.1011942378039299</v>
+      </c>
+      <c r="AA16">
+        <v>180.80896920012299</v>
+      </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2.2499999999999898</v>
       </c>
@@ -3106,32 +5500,55 @@
         <v>2.10396266792208</v>
       </c>
       <c r="D17">
-        <f>1-C17/B17</f>
+        <f t="shared" si="0"/>
         <v>1.7137858538185391E-5</v>
       </c>
       <c r="E17">
         <v>2.1039963023149801</v>
       </c>
       <c r="F17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.151920673736484E-6</v>
       </c>
       <c r="G17">
         <v>2.1039945099552102</v>
       </c>
       <c r="H17">
-        <f>ABS(1-G17/B17)</f>
+        <f t="shared" si="1"/>
         <v>2.0038032094715774E-6</v>
       </c>
       <c r="I17">
         <v>2.1039985842929601</v>
       </c>
       <c r="J17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>6.7329722353015597E-8</v>
       </c>
+      <c r="K17">
+        <v>2.1039955708313798</v>
+      </c>
+      <c r="L17">
+        <v>2.1039986698378699</v>
+      </c>
+      <c r="M17">
+        <f t="shared" si="4"/>
+        <v>1.499584192377057E-6</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="5"/>
+        <v>2.6671470587658064E-8</v>
+      </c>
+      <c r="Y17">
+        <v>2.2499999999999898</v>
+      </c>
+      <c r="Z17">
+        <v>2.1039986698378699</v>
+      </c>
+      <c r="AA17">
+        <v>193.408377600135</v>
+      </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2.25999999999999</v>
       </c>
@@ -3142,32 +5559,55 @@
         <v>2.1068581482015798</v>
       </c>
       <c r="D18">
-        <f>1-C18/B18</f>
+        <f t="shared" si="0"/>
         <v>1.7462189497718938E-5</v>
       </c>
       <c r="E18">
         <v>2.1068922452957901</v>
       </c>
       <c r="F18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.2786135746845062E-6</v>
       </c>
       <c r="G18">
         <v>2.1068897611039401</v>
       </c>
       <c r="H18">
-        <f>ABS(1-G18/B18)</f>
+        <f t="shared" si="1"/>
         <v>2.4576908053131064E-6</v>
       </c>
       <c r="I18">
         <v>2.1068947499033599</v>
       </c>
       <c r="J18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>8.9846387885117451E-8</v>
       </c>
+      <c r="K18">
+        <v>2.10689105943956</v>
+      </c>
+      <c r="L18">
+        <v>2.1068948565283798</v>
+      </c>
+      <c r="M18">
+        <f t="shared" si="4"/>
+        <v>1.8414590247095575E-6</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="5"/>
+        <v>3.9238729265811401E-8</v>
+      </c>
+      <c r="Y18">
+        <v>2.25999999999999</v>
+      </c>
+      <c r="Z18">
+        <v>2.1068948565283798</v>
+      </c>
+      <c r="AA18">
+        <v>206.05378250009301</v>
+      </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2.2699999999999898</v>
       </c>
@@ -3178,32 +5618,55 @@
         <v>2.1098717582622499</v>
       </c>
       <c r="D19">
-        <f>1-C19/B19</f>
+        <f t="shared" si="0"/>
         <v>1.4076735193713219E-5</v>
       </c>
       <c r="E19">
         <v>2.1098992665593501</v>
       </c>
       <c r="F19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.0390186758746367E-6</v>
       </c>
       <c r="G19">
         <v>2.1098951857751098</v>
       </c>
       <c r="H19">
-        <f>ABS(1-G19/B19)</f>
+        <f t="shared" si="1"/>
         <v>2.9731299696633684E-6</v>
       </c>
       <c r="I19">
         <v>2.1099012353718201</v>
       </c>
       <c r="J19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.0588861820703954E-7</v>
       </c>
+      <c r="K19">
+        <v>2.10989621232553</v>
+      </c>
+      <c r="L19">
+        <v>2.1099013448500101</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="4"/>
+        <v>2.4865904605375633E-6</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="5"/>
+        <v>5.4000796834152709E-8</v>
+      </c>
+      <c r="Y19">
+        <v>2.2699999999999898</v>
+      </c>
+      <c r="Z19">
+        <v>2.1099013448500101</v>
+      </c>
+      <c r="AA19">
+        <v>219.12779990001499</v>
+      </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2.27999999999999</v>
       </c>
@@ -3214,33 +5677,56 @@
         <v>2.1130204095340299</v>
       </c>
       <c r="D20">
-        <f>1-C20/B20</f>
+        <f t="shared" si="0"/>
         <v>1.1529645519314791E-5</v>
       </c>
       <c r="E20">
         <v>2.1130431877603599</v>
       </c>
       <c r="F20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>7.4983307529752352E-7</v>
       </c>
       <c r="G20">
         <v>2.1130387643092998</v>
       </c>
       <c r="H20">
-        <f>ABS(1-G20/B20)</f>
+        <f t="shared" si="1"/>
         <v>2.8432345584583629E-6</v>
       </c>
       <c r="I20">
         <v>2.1130446160915701</v>
       </c>
       <c r="J20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>7.3874274586493982E-8</v>
       </c>
+      <c r="K20">
+        <v>2.1130392312680302</v>
+      </c>
+      <c r="L20">
+        <v>2.1130447005506001</v>
+      </c>
+      <c r="M20">
+        <f t="shared" si="4"/>
+        <v>2.6222459942326637E-6</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="5"/>
+        <v>3.3903976182081408E-8</v>
+      </c>
       <c r="O20" s="1"/>
+      <c r="Y20">
+        <v>2.27999999999999</v>
+      </c>
+      <c r="Z20">
+        <v>2.1130447005506001</v>
+      </c>
+      <c r="AA20">
+        <v>232.273500400129</v>
+      </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2.2899999999999898</v>
       </c>
@@ -3251,32 +5737,55 @@
         <v>2.1162707497348299</v>
       </c>
       <c r="D21">
-        <f>1-C21/B21</f>
+        <f t="shared" si="0"/>
         <v>1.0330172572792229E-5</v>
       </c>
       <c r="E21">
         <v>2.1162912433637802</v>
       </c>
       <c r="F21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>6.4643184616297589E-7</v>
       </c>
       <c r="G21">
         <v>2.1162870694923201</v>
       </c>
       <c r="H21">
-        <f>ABS(1-G21/B21)</f>
+        <f t="shared" si="1"/>
         <v>2.618688157762783E-6</v>
       </c>
       <c r="I21">
         <v>2.1162924904658098</v>
       </c>
       <c r="J21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>5.7145646881195944E-8</v>
       </c>
+      <c r="K21">
+        <v>2.1162873157120701</v>
+      </c>
+      <c r="L21">
+        <v>2.1162925589138002</v>
+      </c>
+      <c r="M21">
+        <f t="shared" si="4"/>
+        <v>2.5023433061210909E-6</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="5"/>
+        <v>2.4802297993176126E-8</v>
+      </c>
+      <c r="Y21">
+        <v>2.2899999999999898</v>
+      </c>
+      <c r="Z21">
+        <v>2.1162925589138002</v>
+      </c>
+      <c r="AA21">
+        <v>245.403207800118</v>
+      </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2.2999999999999901</v>
       </c>
@@ -3287,33 +5796,55 @@
         <v>2.11960863439722</v>
       </c>
       <c r="D22">
-        <f>1-C22/B22</f>
+        <f t="shared" si="0"/>
         <v>9.5604489396272641E-6</v>
       </c>
       <c r="E22">
         <v>2.11962766719228</v>
       </c>
       <c r="F22">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>5.8114361456418351E-7</v>
       </c>
       <c r="G22">
         <v>2.1196237999368299</v>
       </c>
       <c r="H22">
-        <f>ABS(1-G22/B22)</f>
+        <f t="shared" si="1"/>
         <v>2.4056400874661321E-6</v>
       </c>
       <c r="I22">
         <v>2.11962879903081</v>
       </c>
       <c r="J22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>4.7164043559533297E-8</v>
       </c>
-      <c r="L22" s="1"/>
+      <c r="K22">
+        <v>2.1196239419329301</v>
+      </c>
+      <c r="L22">
+        <v>2.11962885834892</v>
+      </c>
+      <c r="M22">
+        <f t="shared" si="4"/>
+        <v>2.3386490682897332E-6</v>
+      </c>
+      <c r="N22">
+        <f t="shared" si="5"/>
+        <v>1.9178904353545079E-8</v>
+      </c>
+      <c r="Y22">
+        <v>2.2999999999999901</v>
+      </c>
+      <c r="Z22">
+        <v>2.11962885834892</v>
+      </c>
+      <c r="AA22">
+        <v>258.36892310017703</v>
+      </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2.3099999999999898</v>
       </c>
@@ -3324,34 +5855,56 @@
         <v>2.1230254709324798</v>
       </c>
       <c r="D23">
-        <f>1-C23/B23</f>
+        <f t="shared" si="0"/>
         <v>9.0189965776810155E-6</v>
       </c>
       <c r="E23">
         <v>2.1230434866067198</v>
       </c>
       <c r="F23">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>5.3322379578446544E-7</v>
       </c>
       <c r="G23">
         <v>2.1230400285033499</v>
       </c>
       <c r="H23">
-        <f>ABS(1-G23/B23)</f>
+        <f t="shared" si="1"/>
         <v>2.1620653846143867E-6</v>
       </c>
       <c r="I23">
         <v>2.1230445336498298</v>
       </c>
       <c r="J23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>4.0043812266077339E-8</v>
       </c>
-      <c r="L23" s="1"/>
+      <c r="K23">
+        <v>2.1230400412780601</v>
+      </c>
+      <c r="L23">
+        <v>2.1230445857851801</v>
+      </c>
+      <c r="M23">
+        <f t="shared" si="4"/>
+        <v>2.1560482194038499E-6</v>
+      </c>
+      <c r="N23">
+        <f t="shared" si="5"/>
+        <v>1.5486933069297493E-8</v>
+      </c>
       <c r="O23" s="1"/>
+      <c r="Y23">
+        <v>2.3099999999999898</v>
+      </c>
+      <c r="Z23">
+        <v>2.1230445857851801</v>
+      </c>
+      <c r="AA23">
+        <v>270.07755429996098</v>
+      </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2.3199999999999901</v>
       </c>
@@ -3362,32 +5915,55 @@
         <v>2.1265151145517698</v>
       </c>
       <c r="D24">
-        <f>1-C24/B24</f>
+        <f t="shared" si="0"/>
         <v>8.588626002503652E-6</v>
       </c>
       <c r="E24">
         <v>2.12653232567052</v>
       </c>
       <c r="F24">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>4.9511619737430124E-7</v>
       </c>
       <c r="G24">
         <v>2.1265291389652599</v>
       </c>
       <c r="H24">
-        <f>ABS(1-G24/B24)</f>
+        <f t="shared" si="1"/>
         <v>1.993660867505298E-6</v>
       </c>
       <c r="I24">
         <v>2.12653330539997</v>
       </c>
       <c r="J24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>3.4399493031855854E-8</v>
       </c>
+      <c r="K24">
+        <v>2.12652910626813</v>
+      </c>
+      <c r="L24">
+        <v>2.12653335184145</v>
+      </c>
+      <c r="M24">
+        <f t="shared" si="4"/>
+        <v>2.009036657146801E-6</v>
+      </c>
+      <c r="N24">
+        <f t="shared" si="5"/>
+        <v>1.2560437689934645E-8</v>
+      </c>
+      <c r="Y24">
+        <v>2.3199999999999901</v>
+      </c>
+      <c r="Z24">
+        <v>2.12653335184145</v>
+      </c>
+      <c r="AA24">
+        <v>281.80118059995499</v>
+      </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2.3299999999999899</v>
       </c>
@@ -3398,32 +5974,55 @@
         <v>2.13007262102087</v>
       </c>
       <c r="D25">
-        <f>1-C25/B25</f>
+        <f t="shared" si="0"/>
         <v>8.2579161145845958E-6</v>
       </c>
       <c r="E25">
         <v>2.13008922347711</v>
       </c>
       <c r="F25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>4.6366582728829542E-7</v>
       </c>
       <c r="G25">
         <v>2.1300863033894299</v>
       </c>
       <c r="H25">
-        <f>ABS(1-G25/B25)</f>
+        <f t="shared" si="1"/>
         <v>1.8345409502629195E-6</v>
       </c>
       <c r="I25">
         <v>2.1300901473665701</v>
       </c>
       <c r="J25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.9933276857185831E-8</v>
       </c>
+      <c r="K25">
+        <v>2.1300863146825901</v>
+      </c>
+      <c r="L25">
+        <v>2.1300901889601298</v>
+      </c>
+      <c r="M25">
+        <f t="shared" si="4"/>
+        <v>1.8292392216512354E-6</v>
+      </c>
+      <c r="N25">
+        <f t="shared" si="5"/>
+        <v>1.0406611017366174E-8</v>
+      </c>
+      <c r="Y25">
+        <v>2.3299999999999899</v>
+      </c>
+      <c r="Z25">
+        <v>2.1300901889601298</v>
+      </c>
+      <c r="AA25">
+        <v>293.50468649994502</v>
+      </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2.3399999999999901</v>
       </c>
@@ -3434,32 +6033,55 @@
         <v>2.1336940666666999</v>
       </c>
       <c r="D26">
-        <f>1-C26/B26</f>
+        <f t="shared" si="0"/>
         <v>7.9600973104110295E-6</v>
       </c>
       <c r="E26">
         <v>2.13371012475897</v>
       </c>
       <c r="F26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>4.3419905859654051E-7</v>
       </c>
       <c r="G26">
         <v>2.1337075323717798</v>
       </c>
       <c r="H26">
-        <f>ABS(1-G26/B26)</f>
+        <f t="shared" si="1"/>
         <v>1.6491654378780751E-6</v>
       </c>
       <c r="I26">
         <v>2.1337109955539701</v>
       </c>
       <c r="J26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.6086160898053379E-8</v>
       </c>
+      <c r="K26">
+        <v>2.1337074266531899</v>
+      </c>
+      <c r="L26">
+        <v>2.1337110329732201</v>
+      </c>
+      <c r="M26">
+        <f t="shared" si="4"/>
+        <v>1.6987122543055122E-6</v>
+      </c>
+      <c r="N26">
+        <f t="shared" si="5"/>
+        <v>8.5489925139015099E-9</v>
+      </c>
+      <c r="Y26">
+        <v>2.3399999999999901</v>
+      </c>
+      <c r="Z26">
+        <v>2.1337110329732201</v>
+      </c>
+      <c r="AA26">
+        <v>305.238511400064</v>
+      </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2.3499999999999899</v>
       </c>
@@ -3470,32 +6092,55 @@
         <v>2.1373759349929302</v>
       </c>
       <c r="D27">
-        <f>1-C27/B27</f>
+        <f t="shared" si="0"/>
         <v>7.7309974632067124E-6</v>
       </c>
       <c r="E27">
         <v>2.1373915839917301</v>
       </c>
       <c r="F27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>4.0946007651143645E-7</v>
       </c>
       <c r="G27">
         <v>2.1373893779481699</v>
       </c>
       <c r="H27">
-        <f>ABS(1-G27/B27)</f>
+        <f t="shared" si="1"/>
         <v>1.4415791667055089E-6</v>
       </c>
       <c r="I27">
         <v>2.1373924098081001</v>
       </c>
       <c r="J27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.3093798096063267E-8</v>
       </c>
+      <c r="K27">
+        <v>2.1373891734538799</v>
+      </c>
+      <c r="L27">
+        <v>2.1373924433900302</v>
+      </c>
+      <c r="M27">
+        <f t="shared" si="4"/>
+        <v>1.5372538234581512E-6</v>
+      </c>
+      <c r="N27">
+        <f t="shared" si="5"/>
+        <v>7.3821631030313029E-9</v>
+      </c>
+      <c r="Y27">
+        <v>2.3499999999999899</v>
+      </c>
+      <c r="Z27">
+        <v>2.1373924433900302</v>
+      </c>
+      <c r="AA27">
+        <v>316.91392700001597</v>
+      </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2.3599999999999901</v>
       </c>
@@ -3506,32 +6151,55 @@
         <v>2.14111540495171</v>
       </c>
       <c r="D28">
-        <f>1-C28/B28</f>
+        <f t="shared" si="0"/>
         <v>7.4963739555844455E-6</v>
       </c>
       <c r="E28">
         <v>2.1411306281631002</v>
       </c>
       <c r="F28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>3.8648289790721435E-7</v>
       </c>
       <c r="G28">
         <v>2.1411286298370298</v>
       </c>
       <c r="H28">
-        <f>ABS(1-G28/B28)</f>
+        <f t="shared" si="1"/>
         <v>1.3197866729486307E-6</v>
       </c>
       <c r="I28">
         <v>2.1411314116231202</v>
       </c>
       <c r="J28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>2.0573547532265479E-8</v>
       </c>
+      <c r="K28">
+        <v>2.1411284051890598</v>
+      </c>
+      <c r="L28">
+        <v>2.14113144219422</v>
+      </c>
+      <c r="M28">
+        <f t="shared" si="4"/>
+        <v>1.4247068866879431E-6</v>
+      </c>
+      <c r="N28">
+        <f t="shared" si="5"/>
+        <v>6.2955358703931097E-9</v>
+      </c>
+      <c r="Y28">
+        <v>2.3599999999999901</v>
+      </c>
+      <c r="Z28">
+        <v>2.14113144219422</v>
+      </c>
+      <c r="AA28">
+        <v>328.63836970017201</v>
+      </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2.3699999999999899</v>
       </c>
@@ -3542,32 +6210,55 @@
         <v>2.1449097058861</v>
       </c>
       <c r="D29">
-        <f>1-C29/B29</f>
+        <f t="shared" si="0"/>
         <v>7.3238388386132058E-6</v>
       </c>
       <c r="E29">
         <v>2.1449246285629</v>
       </c>
       <c r="F29">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>3.6663804470205008E-7</v>
       </c>
       <c r="G29">
         <v>2.1449228208168298</v>
       </c>
       <c r="H29">
-        <f>ABS(1-G29/B29)</f>
+        <f t="shared" si="1"/>
         <v>1.2094394108430606E-6</v>
       </c>
       <c r="I29">
         <v>2.1449253754639299</v>
       </c>
       <c r="J29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.8420328262713781E-8</v>
       </c>
+      <c r="K29">
+        <v>2.1449225787020501</v>
+      </c>
+      <c r="L29">
+        <v>2.14492540337974</v>
+      </c>
+      <c r="M29">
+        <f t="shared" si="4"/>
+        <v>1.3223173590537485E-6</v>
+      </c>
+      <c r="N29">
+        <f t="shared" si="5"/>
+        <v>5.4055120379814525E-9</v>
+      </c>
+      <c r="Y29">
+        <v>2.3699999999999899</v>
+      </c>
+      <c r="Z29">
+        <v>2.14492540337974</v>
+      </c>
+      <c r="AA29">
+        <v>340.34521639999002</v>
+      </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2.3799999999999901</v>
       </c>
@@ -3578,32 +6269,55 @@
         <v>2.1487565854628299</v>
       </c>
       <c r="D30">
-        <f>1-C30/B30</f>
+        <f t="shared" si="0"/>
         <v>7.169815815277758E-6</v>
       </c>
       <c r="E30">
         <v>2.1487712466249498</v>
       </c>
       <c r="F30">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>3.4677354920908954E-7</v>
       </c>
       <c r="G30">
         <v>2.1487696110002998</v>
       </c>
       <c r="H30">
-        <f>ABS(1-G30/B30)</f>
+        <f t="shared" si="1"/>
         <v>1.1079639669064889E-6</v>
       </c>
       <c r="I30">
         <v>2.14877195995818</v>
       </c>
       <c r="J30">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.4801039838197028E-8</v>
       </c>
+      <c r="K30">
+        <v>2.1487693519507398</v>
+      </c>
+      <c r="L30">
+        <v>2.1487719817453899</v>
+      </c>
+      <c r="M30">
+        <f t="shared" si="4"/>
+        <v>1.2285209924911555E-6</v>
+      </c>
+      <c r="N30">
+        <f t="shared" si="5"/>
+        <v>4.6616626114825976E-9</v>
+      </c>
+      <c r="Y30">
+        <v>2.3799999999999901</v>
+      </c>
+      <c r="Z30">
+        <v>2.1487719817453899</v>
+      </c>
+      <c r="AA30">
+        <v>352.08665070007498</v>
+      </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2.3899999999999899</v>
       </c>
@@ -3614,32 +6328,55 @@
         <v>2.15265393425579</v>
       </c>
       <c r="D31">
-        <f>1-C31/B31</f>
+        <f t="shared" si="0"/>
         <v>7.0306201818137737E-6</v>
       </c>
       <c r="E31">
         <v>2.1526683620123399</v>
       </c>
       <c r="F31">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>3.2835611407655563E-7</v>
       </c>
       <c r="G31">
         <v>2.15266688623699</v>
       </c>
       <c r="H31">
-        <f>ABS(1-G31/B31)</f>
+        <f t="shared" si="1"/>
         <v>1.0139121854324529E-6</v>
       </c>
       <c r="I31">
         <v>2.1526690401144601</v>
       </c>
       <c r="J31">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.3350835215142354E-8</v>
       </c>
+      <c r="K31">
+        <v>2.15266668009125</v>
+      </c>
+      <c r="L31">
+        <v>2.15266906013027</v>
+      </c>
+      <c r="M31">
+        <f t="shared" si="4"/>
+        <v>1.1096750424099966E-6</v>
+      </c>
+      <c r="N31">
+        <f t="shared" si="5"/>
+        <v>4.0526991762490638E-9</v>
+      </c>
+      <c r="Y31">
+        <v>2.3899999999999899</v>
+      </c>
+      <c r="Z31">
+        <v>2.15266906013027</v>
+      </c>
+      <c r="AA31">
+        <v>363.76235319999898</v>
+      </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2.3999999999999901</v>
       </c>
@@ -3650,32 +6387,55 @@
         <v>2.15659983030779</v>
       </c>
       <c r="D32">
-        <f>1-C32/B32</f>
+        <f t="shared" si="0"/>
         <v>6.9034626550834588E-6</v>
       </c>
       <c r="E32">
         <v>2.1566140490429202</v>
       </c>
       <c r="F32">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>3.1038183778697714E-7</v>
       </c>
       <c r="G32">
         <v>2.1566127202490799</v>
       </c>
       <c r="H32">
-        <f>ABS(1-G32/B32)</f>
+        <f t="shared" si="1"/>
         <v>9.2652983540997269E-7</v>
       </c>
       <c r="I32">
         <v>2.1566146923749501</v>
       </c>
       <c r="J32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.2075411337519881E-8</v>
       </c>
+      <c r="K32">
+        <v>2.1566124991445901</v>
+      </c>
+      <c r="L32">
+        <v>2.15661471077133</v>
+      </c>
+      <c r="M32">
+        <f t="shared" si="4"/>
+        <v>1.0290537066914851E-6</v>
+      </c>
+      <c r="N32">
+        <f t="shared" si="5"/>
+        <v>3.5451996893698379E-9</v>
+      </c>
+      <c r="Y32">
+        <v>2.3999999999999901</v>
+      </c>
+      <c r="Z32">
+        <v>2.15661471077133</v>
+      </c>
+      <c r="AA32">
+        <v>375.513260500039</v>
+      </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2.4099999999999899</v>
       </c>
@@ -3686,32 +6446,55 @@
         <v>2.1605925846730298</v>
       </c>
       <c r="D33">
-        <f>1-C33/B33</f>
+        <f t="shared" si="0"/>
         <v>6.7516846173898415E-6</v>
       </c>
       <c r="E33">
         <v>2.1606065355508699</v>
       </c>
       <c r="F33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.9475990748206726E-7</v>
       </c>
       <c r="G33">
         <v>2.1606053458178902</v>
       </c>
       <c r="H33">
-        <f>ABS(1-G33/B33)</f>
+        <f t="shared" si="1"/>
         <v>8.4540742673056002E-7</v>
       </c>
       <c r="I33">
         <v>2.16060714873313</v>
       </c>
       <c r="J33">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.0959007479272032E-8</v>
       </c>
+      <c r="K33">
+        <v>2.1606051068434402</v>
+      </c>
+      <c r="L33">
+        <v>2.16060716567964</v>
+      </c>
+      <c r="M33">
+        <f t="shared" si="4"/>
+        <v>9.5601265526212842E-7</v>
+      </c>
+      <c r="N33">
+        <f t="shared" si="5"/>
+        <v>3.1156057733738862E-9</v>
+      </c>
+      <c r="Y33">
+        <v>2.4099999999999899</v>
+      </c>
+      <c r="Z33">
+        <v>2.16060716567964</v>
+      </c>
+      <c r="AA33">
+        <v>386.72877630009299</v>
+      </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2.4199999999999902</v>
       </c>
@@ -3722,32 +6505,55 @@
         <v>2.1646304166716099</v>
       </c>
       <c r="D34">
-        <f>1-C34/B34</f>
+        <f t="shared" si="0"/>
         <v>6.6444440969259944E-6</v>
       </c>
       <c r="E34">
         <v>2.1646441908779601</v>
       </c>
       <c r="F34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.811800855484492E-7</v>
       </c>
       <c r="G34">
         <v>2.16464319824955</v>
       </c>
       <c r="H34">
-        <f>ABS(1-G34/B34)</f>
+        <f t="shared" si="1"/>
         <v>7.3974419290134819E-7</v>
       </c>
       <c r="I34">
         <v>2.16464477793579</v>
       </c>
       <c r="J34">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>9.9772397010866598E-9</v>
       </c>
+      <c r="K34">
+        <v>2.16464287411769</v>
+      </c>
+      <c r="L34">
+        <v>2.1646447935723501</v>
+      </c>
+      <c r="M34">
+        <f t="shared" si="4"/>
+        <v>8.8948324483695274E-7</v>
+      </c>
+      <c r="N34">
+        <f t="shared" si="5"/>
+        <v>2.7536249946891189E-9</v>
+      </c>
+      <c r="Y34">
+        <v>2.4199999999999902</v>
+      </c>
+      <c r="Z34">
+        <v>2.1646447935723501</v>
+      </c>
+      <c r="AA34">
+        <v>398.04589310008998</v>
+      </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2.4299999999999899</v>
       </c>
@@ -3758,32 +6564,55 @@
         <v>2.1687118925606499</v>
       </c>
       <c r="D35">
-        <f>1-C35/B35</f>
+        <f t="shared" si="0"/>
         <v>6.5449949839813115E-6</v>
       </c>
       <c r="E35">
         <v>2.1687255074642802</v>
       </c>
       <c r="F35">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.6716040046892431E-7</v>
       </c>
       <c r="G35">
         <v>2.1687246302613801</v>
       </c>
       <c r="H35">
-        <f>ABS(1-G35/B35)</f>
+        <f t="shared" si="1"/>
         <v>6.7163882000453867E-7</v>
       </c>
       <c r="I35">
         <v>2.1687260671018</v>
       </c>
       <c r="J35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>9.1114364941802251E-9</v>
       </c>
+      <c r="K35">
+        <v>2.16872428986705</v>
+      </c>
+      <c r="L35">
+        <v>2.1687260815512701</v>
+      </c>
+      <c r="M35">
+        <f t="shared" si="4"/>
+        <v>8.2859470862395312E-7</v>
+      </c>
+      <c r="N35">
+        <f t="shared" si="5"/>
+        <v>2.4487831762343149E-9</v>
+      </c>
+      <c r="Y35">
+        <v>2.4299999999999899</v>
+      </c>
+      <c r="Z35">
+        <v>2.1687260815512701</v>
+      </c>
+      <c r="AA35">
+        <v>409.26210750010699</v>
+      </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2.4399999999999902</v>
       </c>
@@ -3794,32 +6623,55 @@
         <v>2.1728356052905702</v>
       </c>
       <c r="D36">
-        <f>1-C36/B36</f>
+        <f t="shared" si="0"/>
         <v>6.4522285291301884E-6</v>
       </c>
       <c r="E36">
         <v>2.1728490729575398</v>
       </c>
       <c r="F36">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.5406975423525324E-7</v>
       </c>
       <c r="G36">
         <v>2.17284830144049</v>
       </c>
       <c r="H36">
-        <f>ABS(1-G36/B36)</f>
+        <f t="shared" si="1"/>
         <v>6.0914128841016435E-7</v>
       </c>
       <c r="I36">
         <v>2.17284960688563</v>
       </c>
       <c r="J36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>8.342629809199309E-9</v>
       </c>
+      <c r="K36">
+        <v>2.1728479462723702</v>
+      </c>
+      <c r="L36">
+        <v>2.1728496202565002</v>
+      </c>
+      <c r="M36">
+        <f t="shared" si="4"/>
+        <v>7.7259858233258427E-7</v>
+      </c>
+      <c r="N36">
+        <f t="shared" si="5"/>
+        <v>2.1890194101814586E-9</v>
+      </c>
+      <c r="Y36">
+        <v>2.4399999999999902</v>
+      </c>
+      <c r="Z36">
+        <v>2.1728496202565002</v>
+      </c>
+      <c r="AA36">
+        <v>420.56664249999397</v>
+      </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2.44999999999999</v>
       </c>
@@ -3830,32 +6682,55 @@
         <v>2.1770002387688199</v>
       </c>
       <c r="D37">
-        <f>1-C37/B37</f>
+        <f t="shared" si="0"/>
         <v>6.3652202786368406E-6</v>
       </c>
       <c r="E37">
         <v>2.1770135694813399</v>
       </c>
       <c r="F37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.4182744207124074E-7</v>
       </c>
       <c r="G37">
         <v>2.1770128962034798</v>
       </c>
       <c r="H37">
-        <f>ABS(1-G37/B37)</f>
+        <f t="shared" si="1"/>
         <v>5.5109409380360574E-7</v>
       </c>
       <c r="I37">
         <v>2.1770140789644299</v>
       </c>
       <c r="J37">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>7.7990585101161969E-9</v>
       </c>
+      <c r="K37">
+        <v>2.1770125612645299</v>
+      </c>
+      <c r="L37">
+        <v>2.1770140917102401</v>
+      </c>
+      <c r="M37">
+        <f t="shared" si="4"/>
+        <v>7.0494654269559476E-7</v>
+      </c>
+      <c r="N37">
+        <f t="shared" si="5"/>
+        <v>1.9443374688066228E-9</v>
+      </c>
+      <c r="Y37">
+        <v>2.44999999999999</v>
+      </c>
+      <c r="Z37">
+        <v>2.1770140917102401</v>
+      </c>
+      <c r="AA37">
+        <v>431.78228299994902</v>
+      </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2.4599999999999902</v>
       </c>
@@ -3866,32 +6741,55 @@
         <v>2.1812045578259802</v>
       </c>
       <c r="D38">
-        <f>1-C38/B38</f>
+        <f t="shared" si="0"/>
         <v>6.2831811622476863E-6</v>
       </c>
       <c r="E38">
         <v>2.1812177603469101</v>
       </c>
       <c r="F38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.3036143537158438E-7</v>
       </c>
       <c r="G38">
         <v>2.1812172333990798</v>
       </c>
       <c r="H38">
-        <f>ABS(1-G38/B38)</f>
+        <f t="shared" si="1"/>
         <v>4.7194561758612252E-7</v>
       </c>
       <c r="I38">
         <v>2.18121824712766</v>
       </c>
       <c r="J38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>7.1922283684244803E-9</v>
       </c>
+      <c r="K38">
+        <v>2.1812168334379698</v>
+      </c>
+      <c r="L38">
+        <v>2.1812182589979199</v>
+      </c>
+      <c r="M38">
+        <f t="shared" si="4"/>
+        <v>6.5531154513909229E-7</v>
+      </c>
+      <c r="N38">
+        <f t="shared" si="5"/>
+        <v>1.7501962101817981E-9</v>
+      </c>
+      <c r="Y38">
+        <v>2.4599999999999902</v>
+      </c>
+      <c r="Z38">
+        <v>2.1812182589979199</v>
+      </c>
+      <c r="AA38">
+        <v>443.09683239995502</v>
+      </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2.46999999999999</v>
       </c>
@@ -3902,32 +6800,55 @@
         <v>2.1854473997669599</v>
       </c>
       <c r="D39">
-        <f>1-C39/B39</f>
+        <f t="shared" si="0"/>
         <v>6.2054222514928981E-6</v>
       </c>
       <c r="E39">
         <v>2.1854604815330401</v>
       </c>
       <c r="F39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.196067595550133E-7</v>
       </c>
       <c r="G39">
         <v>2.18546003800749</v>
       </c>
       <c r="H39">
-        <f>ABS(1-G39/B39)</f>
+        <f t="shared" si="1"/>
         <v>4.2255046706074495E-7</v>
       </c>
       <c r="I39">
         <v>2.18546094704887</v>
       </c>
       <c r="J39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>6.6009735455452301E-9</v>
       </c>
+      <c r="K39">
+        <v>2.18545962783723</v>
+      </c>
+      <c r="L39">
+        <v>2.1854609580574502</v>
+      </c>
+      <c r="M39">
+        <f t="shared" si="4"/>
+        <v>6.1023181541219884E-7</v>
+      </c>
+      <c r="N39">
+        <f t="shared" si="5"/>
+        <v>1.5637844352767161E-9</v>
+      </c>
+      <c r="Y39">
+        <v>2.46999999999999</v>
+      </c>
+      <c r="Z39">
+        <v>2.1854609580574502</v>
+      </c>
+      <c r="AA39">
+        <v>454.34593560011098</v>
+      </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2.4799999999999902</v>
       </c>
@@ -3938,32 +6859,55 @@
         <v>2.1897277453742801</v>
       </c>
       <c r="D40">
-        <f>1-C40/B40</f>
+        <f t="shared" si="0"/>
         <v>6.0956233050024622E-6</v>
       </c>
       <c r="E40">
         <v>2.1897406344485599</v>
       </c>
       <c r="F40">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.0950538914821237E-7</v>
       </c>
       <c r="G40">
         <v>2.1897402656619001</v>
       </c>
       <c r="H40">
-        <f>ABS(1-G40/B40)</f>
+        <f t="shared" si="1"/>
         <v>3.7792103479983297E-7</v>
       </c>
       <c r="I40">
         <v>2.18974107949037</v>
       </c>
       <c r="J40">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>6.2659233357464927E-9</v>
       </c>
+      <c r="K40">
+        <v>2.1897398469156699</v>
+      </c>
+      <c r="L40">
+        <v>2.1897410901102998</v>
+      </c>
+      <c r="M40">
+        <f t="shared" si="4"/>
+        <v>5.6915196677831403E-7</v>
+      </c>
+      <c r="N40">
+        <f t="shared" si="5"/>
+        <v>1.4160669303819873E-9</v>
+      </c>
+      <c r="Y40">
+        <v>2.4799999999999902</v>
+      </c>
+      <c r="Z40">
+        <v>2.1897410901102998</v>
+      </c>
+      <c r="AA40">
+        <v>465.72668020008098</v>
+      </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2.48999999999999</v>
       </c>
@@ -3974,32 +6918,55 @@
         <v>2.1940444031437298</v>
       </c>
       <c r="D41">
-        <f>1-C41/B41</f>
+        <f t="shared" si="0"/>
         <v>6.0232755140221528E-6</v>
       </c>
       <c r="E41">
         <v>2.1940571806306299</v>
       </c>
       <c r="F41">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.9959668617897108E-7</v>
       </c>
       <c r="G41">
         <v>2.19405711459593</v>
       </c>
       <c r="H41">
-        <f>ABS(1-G41/B41)</f>
+        <f t="shared" si="1"/>
         <v>2.2969375357284605E-7</v>
       </c>
       <c r="I41">
         <v>2.1940576057940699</v>
       </c>
       <c r="J41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>5.8171626404757149E-9</v>
       </c>
+      <c r="K41">
+        <v>2.19405645220399</v>
+      </c>
+      <c r="L41">
+        <v>2.1940576157332701</v>
+      </c>
+      <c r="M41">
+        <f t="shared" si="4"/>
+        <v>5.315964631824599E-7</v>
+      </c>
+      <c r="N41">
+        <f t="shared" si="5"/>
+        <v>1.2871084198451399E-9</v>
+      </c>
+      <c r="Y41">
+        <v>2.48999999999999</v>
+      </c>
+      <c r="Z41">
+        <v>2.1940576157332701</v>
+      </c>
+      <c r="AA41">
+        <v>477.02889199997298</v>
+      </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2.4999999999999898</v>
       </c>
@@ -4010,29 +6977,52 @@
         <v>2.1983964615488198</v>
       </c>
       <c r="D42">
-        <f>1-C42/B42</f>
+        <f t="shared" si="0"/>
         <v>5.9544812879286368E-6</v>
       </c>
       <c r="E42">
         <v>2.1984091325937598</v>
       </c>
       <c r="F42">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.9074862545043203E-7</v>
       </c>
       <c r="G42">
         <v>2.1984091166872402</v>
       </c>
       <c r="H42">
-        <f>ABS(1-G42/B42)</f>
+        <f t="shared" si="1"/>
         <v>1.9798409245375126E-7</v>
       </c>
       <c r="I42">
         <v>2.1984095712593099</v>
       </c>
       <c r="J42">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>8.7890583699845592E-9</v>
+      </c>
+      <c r="K42">
+        <v>2.1984084589766901</v>
+      </c>
+      <c r="L42">
+        <v>2.1984095493616098</v>
+      </c>
+      <c r="M42">
+        <f t="shared" si="4"/>
+        <v>4.9715971661701275E-7</v>
+      </c>
+      <c r="N42">
+        <f t="shared" si="5"/>
+        <v>1.1716425607488645E-9</v>
+      </c>
+      <c r="Y42">
+        <v>2.4999999999999898</v>
+      </c>
+      <c r="Z42">
+        <v>2.1984095493616098</v>
+      </c>
+      <c r="AA42">
+        <v>489.29462349996902</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correction for BTRG. Graphs were updated.
</commit_message>
<xml_diff>
--- a/Additional/Tests.xlsx
+++ b/Additional/Tests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iakob\Desktop\programing\tensornetworks\Additional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1169C9B7-FA8E-4EB4-B984-83E45CA624B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{393F3F7F-70EB-4247-90ED-A07DB2A6B94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4E5A4C81-6162-4430-A263-13FAAFDD787D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{4E5A4C81-6162-4430-A263-13FAAFDD787D}"/>
   </bookViews>
   <sheets>
     <sheet name="Ising_compare" sheetId="1" r:id="rId1"/>
@@ -4288,49 +4288,49 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="121"/>
                 <c:pt idx="0">
-                  <c:v>1.4643841694805815E-13</c:v>
+                  <c:v>1.7508217098338719E-13</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.0412118096355698E-14</c:v>
+                  <c:v>5.1514348342607263E-14</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.4386716524513758E-13</c:v>
+                  <c:v>4.2721381987576024E-13</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.4710016778899444E-14</c:v>
+                  <c:v>5.7398530373120593E-14</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.1078251911130792E-14</c:v>
+                  <c:v>1.9317880628477724E-14</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.9118040484045196E-13</c:v>
+                  <c:v>1.8873791418627661E-13</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>8.8817841970012523E-15</c:v>
+                  <c:v>1.3433698597964394E-14</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.7108536809473662E-13</c:v>
+                  <c:v>1.6298074001497298E-13</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.9531932455029164E-14</c:v>
+                  <c:v>1.1324274851176597E-14</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5.5289106626332796E-14</c:v>
+                  <c:v>6.1950444774083735E-14</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>6.3726801613483985E-14</c:v>
+                  <c:v>5.4622972811557702E-14</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>5.5511151231257827E-15</c:v>
+                  <c:v>9.7699626167013776E-15</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.7525538232330291E-14</c:v>
+                  <c:v>4.3742787170231168E-14</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.6193270602780103E-14</c:v>
+                  <c:v>3.1641356201816961E-14</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2.7866597918091429E-14</c:v>
+                  <c:v>2.5757174171303632E-14</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>0</c:v>
@@ -4339,40 +4339,40 @@
                   <c:v>8.5487172896137054E-15</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3.8413716652030416E-14</c:v>
+                  <c:v>3.0864200084579352E-14</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>7.1054273576010019E-15</c:v>
+                  <c:v>1.4099832412739488E-14</c:v>
                 </c:pt>
                 <c:pt idx="19">
                   <c:v>6.4392935428259079E-15</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1.1546319456101628E-14</c:v>
+                  <c:v>1.7319479184152442E-14</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>7.9047879353311146E-14</c:v>
+                  <c:v>7.382983113757291E-14</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>4.8849813083506888E-15</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>4.3742787170231168E-14</c:v>
+                  <c:v>4.8183679268731794E-14</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>3.1974423109204508E-14</c:v>
+                  <c:v>2.7977620220553945E-14</c:v>
                 </c:pt>
                 <c:pt idx="25">
                   <c:v>1.8207657603852567E-14</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1.3322676295501878E-14</c:v>
+                  <c:v>1.6653345369377348E-14</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>3.0420110874729289E-14</c:v>
+                  <c:v>3.3528735343679728E-14</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>5.5511151231257827E-15</c:v>
+                  <c:v>8.2156503822261584E-15</c:v>
                 </c:pt>
                 <c:pt idx="29">
                   <c:v>7.5495165674510645E-15</c:v>
@@ -4381,34 +4381,34 @@
                   <c:v>2.2204460492503131E-15</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1.4988010832439613E-14</c:v>
+                  <c:v>1.7208456881689926E-14</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1.5765166949677223E-14</c:v>
+                  <c:v>1.3766765505351941E-14</c:v>
                 </c:pt>
                 <c:pt idx="33">
                   <c:v>8.992806499463768E-15</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>9.9920072216264089E-15</c:v>
+                  <c:v>1.1657341758564144E-14</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>2.4313884239290928E-14</c:v>
+                  <c:v>2.5868196473766147E-14</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>5.6621374255882984E-15</c:v>
+                  <c:v>4.3298697960381105E-15</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>6.4392935428259079E-15</c:v>
+                  <c:v>7.7715611723760958E-15</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>2.3980817331903381E-14</c:v>
+                  <c:v>2.5202062658991053E-14</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>1.4432899320127035E-14</c:v>
+                  <c:v>1.532107773982716E-14</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>2.0650148258027912E-14</c:v>
+                  <c:v>1.9539925233402755E-14</c:v>
                 </c:pt>
                 <c:pt idx="41">
                   <c:v>4.7961634663806763E-14</c:v>
@@ -4444,7 +4444,7 @@
                   <c:v>4.8841375388519737E-11</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>7.2251316041160862E-11</c:v>
+                  <c:v>7.2246653104457437E-11</c:v>
                 </c:pt>
                 <c:pt idx="53">
                   <c:v>1.1031686675266883E-10</c:v>
@@ -4456,7 +4456,7 @@
                   <c:v>2.1678658868040657E-10</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>2.7060376162069133E-10</c:v>
+                  <c:v>2.7060020890701253E-10</c:v>
                 </c:pt>
                 <c:pt idx="57">
                   <c:v>2.9727109662758266E-10</c:v>
@@ -4465,13 +4465,13 @@
                   <c:v>2.5259705438429592E-10</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>6.3737237709915462E-11</c:v>
+                  <c:v>6.3740568378989337E-11</c:v>
                 </c:pt>
                 <c:pt idx="60">
                   <c:v>3.8204883701098424E-10</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>1.2580219088675904E-9</c:v>
+                  <c:v>1.2580190222877263E-9</c:v>
                 </c:pt>
                 <c:pt idx="62">
                   <c:v>2.7802863344916773E-9</c:v>
@@ -4492,7 +4492,7 @@
                   <c:v>2.4592849423576979E-8</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>3.5383043939241077E-8</c:v>
+                  <c:v>3.5383046048664824E-8</c:v>
                 </c:pt>
                 <c:pt idx="69">
                   <c:v>4.9790182310438524E-8</c:v>
@@ -4522,7 +4522,7 @@
                   <c:v>3.1275613654457857E-8</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>1.6161475580034335E-7</c:v>
+                  <c:v>1.6161475446807572E-7</c:v>
                 </c:pt>
                 <c:pt idx="79">
                   <c:v>3.149945406732968E-7</c:v>
@@ -4531,124 +4531,124 @@
                   <c:v>6.000734524835849E-7</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>1.0019068330535674E-6</c:v>
+                  <c:v>1.0019068421573962E-6</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>1.9248254703452261E-6</c:v>
+                  <c:v>1.9248254805592779E-6</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>2.1904909046632781E-6</c:v>
+                  <c:v>2.1904909146552853E-6</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>2.2010848779174808E-6</c:v>
+                  <c:v>2.2010848874653988E-6</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>2.6814328810687016E-6</c:v>
+                  <c:v>2.6814318661028125E-6</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>2.6305790117309158E-6</c:v>
+                  <c:v>2.6305778222379672E-6</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>2.3824640933423069E-6</c:v>
+                  <c:v>2.3822487731361974E-6</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>2.0172683945496317E-6</c:v>
+                  <c:v>2.0173012860169592E-6</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>1.6596062042406601E-6</c:v>
+                  <c:v>1.6603655250690963E-6</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>1.4557962801919899E-6</c:v>
+                  <c:v>1.4557959757688366E-6</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>4.4216355914450389E-6</c:v>
+                  <c:v>1.2084340144102867E-6</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>9.7852029257161632E-7</c:v>
+                  <c:v>9.793573605421102E-7</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>7.7933714193179071E-7</c:v>
+                  <c:v>7.793238456788032E-7</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>6.0827867232049471E-7</c:v>
+                  <c:v>6.0759494724393903E-7</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>4.6622668414819657E-7</c:v>
+                  <c:v>4.6623229899012131E-7</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>1.3997863690384804E-6</c:v>
+                  <c:v>3.504052046299222E-7</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>1.1089460489888125E-6</c:v>
+                  <c:v>2.5886858057155848E-7</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>1.9035024534375111E-7</c:v>
+                  <c:v>1.9036906206970627E-7</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>1.4015218607887903E-7</c:v>
+                  <c:v>1.4015685345647455E-7</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>1.0215985923878179E-7</c:v>
+                  <c:v>1.0221056023773656E-7</c:v>
                 </c:pt>
                 <c:pt idx="101">
-                  <c:v>6.329168145136066E-8</c:v>
+                  <c:v>7.3875976225323825E-8</c:v>
                 </c:pt>
                 <c:pt idx="102">
-                  <c:v>4.3287819107007408E-8</c:v>
+                  <c:v>5.2978468056963379E-8</c:v>
                 </c:pt>
                 <c:pt idx="103">
-                  <c:v>3.7269541897089198E-8</c:v>
+                  <c:v>3.4761274969596911E-8</c:v>
                 </c:pt>
                 <c:pt idx="104">
-                  <c:v>2.6611679970756086E-8</c:v>
+                  <c:v>2.6109435724563923E-8</c:v>
                 </c:pt>
                 <c:pt idx="105">
-                  <c:v>1.8128855527876908E-8</c:v>
+                  <c:v>1.8558363512610754E-8</c:v>
                 </c:pt>
                 <c:pt idx="106">
-                  <c:v>1.3884142702202951E-7</c:v>
+                  <c:v>1.2602239696235529E-8</c:v>
                 </c:pt>
                 <c:pt idx="107">
-                  <c:v>8.918725091788815E-9</c:v>
+                  <c:v>8.8829101851928272E-9</c:v>
                 </c:pt>
                 <c:pt idx="108">
-                  <c:v>5.3184776582781979E-9</c:v>
+                  <c:v>5.9951841269167971E-9</c:v>
                 </c:pt>
                 <c:pt idx="109">
-                  <c:v>3.9748777602710561E-9</c:v>
+                  <c:v>4.4149564004669628E-9</c:v>
                 </c:pt>
                 <c:pt idx="110">
-                  <c:v>2.147691802178997E-9</c:v>
+                  <c:v>2.6033712963169364E-9</c:v>
                 </c:pt>
                 <c:pt idx="111">
-                  <c:v>1.2598797560769981E-9</c:v>
+                  <c:v>5.9563483034708042E-9</c:v>
                 </c:pt>
                 <c:pt idx="112">
-                  <c:v>1.0405907246990864E-9</c:v>
+                  <c:v>5.5443560853518647E-10</c:v>
                 </c:pt>
                 <c:pt idx="113">
-                  <c:v>2.8937487739355561E-8</c:v>
+                  <c:v>5.010902803803674E-11</c:v>
                 </c:pt>
                 <c:pt idx="114">
-                  <c:v>3.3152636191857709E-10</c:v>
+                  <c:v>1.9412540464003314E-9</c:v>
                 </c:pt>
                 <c:pt idx="115">
-                  <c:v>3.9087499903445178E-10</c:v>
+                  <c:v>1.7866597090687719E-11</c:v>
                 </c:pt>
                 <c:pt idx="116">
-                  <c:v>4.5296655315496537E-11</c:v>
+                  <c:v>3.4969582785038256E-11</c:v>
                 </c:pt>
                 <c:pt idx="117">
-                  <c:v>2.421587153023097E-9</c:v>
+                  <c:v>1.8404944235328458E-11</c:v>
                 </c:pt>
                 <c:pt idx="118">
-                  <c:v>5.197098307263559E-11</c:v>
+                  <c:v>9.1963769932590367E-11</c:v>
                 </c:pt>
                 <c:pt idx="119">
-                  <c:v>9.6163632612444871E-11</c:v>
+                  <c:v>2.174403213039966E-9</c:v>
                 </c:pt>
                 <c:pt idx="120">
-                  <c:v>6.5787597591793201E-11</c:v>
+                  <c:v>6.5817795658063005E-11</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6963,20 +6963,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7195F39-8342-4B20-915A-AACA967BE21D}">
   <dimension ref="A1:AA42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="12.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" customWidth="1"/>
-    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" customWidth="1"/>
-    <col min="9" max="9" width="10.42578125" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.109375" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="10" max="10" width="14.5546875" customWidth="1"/>
+    <col min="13" max="13" width="13.88671875" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -7020,7 +7020,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2.1</v>
       </c>
@@ -7079,7 +7079,7 @@
         <v>10.822773599997101</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2.11</v>
       </c>
@@ -7138,7 +7138,7 @@
         <v>22.873911099973999</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2.1199999999999899</v>
       </c>
@@ -7197,7 +7197,7 @@
         <v>34.9319418000523</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2.1299999999999901</v>
       </c>
@@ -7256,7 +7256,7 @@
         <v>46.990211399970498</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2.1399999999999899</v>
       </c>
@@ -7315,7 +7315,7 @@
         <v>59.067980400053699</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2.1499999999999901</v>
       </c>
@@ -7374,7 +7374,7 @@
         <v>71.139418700011404</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2.1599999999999899</v>
       </c>
@@ -7433,7 +7433,7 @@
         <v>83.186399300117003</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2.1699999999999902</v>
       </c>
@@ -7492,7 +7492,7 @@
         <v>95.245498999953199</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2.1799999999999899</v>
       </c>
@@ -7551,7 +7551,7 @@
         <v>107.29150560009199</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2.1899999999999902</v>
       </c>
@@ -7610,7 +7610,7 @@
         <v>119.347242100164</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2.19999999999999</v>
       </c>
@@ -7669,7 +7669,7 @@
         <v>131.420531400013</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2.2099999999999902</v>
       </c>
@@ -7728,7 +7728,7 @@
         <v>143.49993579997599</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2.21999999999999</v>
       </c>
@@ -7787,7 +7787,7 @@
         <v>155.588994800113</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2.2299999999999902</v>
       </c>
@@ -7846,7 +7846,7 @@
         <v>168.195618000114</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2.23999999999999</v>
       </c>
@@ -7905,7 +7905,7 @@
         <v>180.80896920012299</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2.2499999999999898</v>
       </c>
@@ -7964,7 +7964,7 @@
         <v>193.408377600135</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2.25999999999999</v>
       </c>
@@ -8023,7 +8023,7 @@
         <v>206.05378250009301</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2.2699999999999898</v>
       </c>
@@ -8082,7 +8082,7 @@
         <v>219.12779990001499</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2.27999999999999</v>
       </c>
@@ -8142,7 +8142,7 @@
         <v>232.273500400129</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2.2899999999999898</v>
       </c>
@@ -8201,7 +8201,7 @@
         <v>245.403207800118</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2.2999999999999901</v>
       </c>
@@ -8260,7 +8260,7 @@
         <v>258.36892310017703</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2.3099999999999898</v>
       </c>
@@ -8320,7 +8320,7 @@
         <v>270.07755429996098</v>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2.3199999999999901</v>
       </c>
@@ -8379,7 +8379,7 @@
         <v>281.80118059995499</v>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2.3299999999999899</v>
       </c>
@@ -8438,7 +8438,7 @@
         <v>293.50468649994502</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2.3399999999999901</v>
       </c>
@@ -8497,7 +8497,7 @@
         <v>305.238511400064</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2.3499999999999899</v>
       </c>
@@ -8556,7 +8556,7 @@
         <v>316.91392700001597</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2.3599999999999901</v>
       </c>
@@ -8615,7 +8615,7 @@
         <v>328.63836970017201</v>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>2.3699999999999899</v>
       </c>
@@ -8674,7 +8674,7 @@
         <v>340.34521639999002</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>2.3799999999999901</v>
       </c>
@@ -8733,7 +8733,7 @@
         <v>352.08665070007498</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>2.3899999999999899</v>
       </c>
@@ -8792,7 +8792,7 @@
         <v>363.76235319999898</v>
       </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>2.3999999999999901</v>
       </c>
@@ -8851,7 +8851,7 @@
         <v>375.513260500039</v>
       </c>
     </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>2.4099999999999899</v>
       </c>
@@ -8910,7 +8910,7 @@
         <v>386.72877630009299</v>
       </c>
     </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>2.4199999999999902</v>
       </c>
@@ -8969,7 +8969,7 @@
         <v>398.04589310008998</v>
       </c>
     </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>2.4299999999999899</v>
       </c>
@@ -9028,7 +9028,7 @@
         <v>409.26210750010699</v>
       </c>
     </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>2.4399999999999902</v>
       </c>
@@ -9087,7 +9087,7 @@
         <v>420.56664249999397</v>
       </c>
     </row>
-    <row r="37" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>2.44999999999999</v>
       </c>
@@ -9146,7 +9146,7 @@
         <v>431.78228299994902</v>
       </c>
     </row>
-    <row r="38" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>2.4599999999999902</v>
       </c>
@@ -9205,7 +9205,7 @@
         <v>443.09683239995502</v>
       </c>
     </row>
-    <row r="39" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>2.46999999999999</v>
       </c>
@@ -9264,7 +9264,7 @@
         <v>454.34593560011098</v>
       </c>
     </row>
-    <row r="40" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>2.4799999999999902</v>
       </c>
@@ -9323,7 +9323,7 @@
         <v>465.72668020008098</v>
       </c>
     </row>
-    <row r="41" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>2.48999999999999</v>
       </c>
@@ -9382,7 +9382,7 @@
         <v>477.02889199997298</v>
       </c>
     </row>
-    <row r="42" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>2.4999999999999898</v>
       </c>
@@ -9450,14 +9450,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1368E99-E726-48A5-9354-F032CB1ADBEA}">
-  <dimension ref="A1:H122"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I122"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="13.85546875" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -9477,7 +9477,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>-6</v>
       </c>
@@ -9492,14 +9492,14 @@
         <v>1.9129142714291447E-13</v>
       </c>
       <c r="E2">
-        <v>2.4575370705772902E-3</v>
+        <v>2.4575370705772199E-3</v>
       </c>
       <c r="F2">
         <f>ABS(1-E2/B2)</f>
-        <v>1.4643841694805815E-13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.7508217098338719E-13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>-5.9</v>
       </c>
@@ -9514,14 +9514,14 @@
         <v>5.5289106626332796E-14</v>
       </c>
       <c r="E3">
-        <v>2.7135691662694599E-3</v>
+        <v>2.7135691662694898E-3</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F67" si="1">ABS(1-E3/B3)</f>
-        <v>4.0412118096355698E-14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>5.1514348342607263E-14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>-5.8</v>
       </c>
@@ -9536,14 +9536,14 @@
         <v>2.3026025530725747E-13</v>
       </c>
       <c r="E4">
-        <v>2.9959992943517102E-3</v>
+        <v>2.9959992943516599E-3</v>
       </c>
       <c r="F4">
         <f t="shared" si="1"/>
-        <v>4.4386716524513758E-13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4.2721381987576024E-13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>-5.7</v>
       </c>
@@ -9558,14 +9558,14 @@
         <v>1.7530421558831222E-13</v>
       </c>
       <c r="E5">
-        <v>3.3074896154375198E-3</v>
+        <v>3.30748961543761E-3</v>
       </c>
       <c r="F5">
         <f t="shared" si="1"/>
-        <v>8.4710016778899444E-14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>5.7398530373120593E-14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>-5.6</v>
       </c>
@@ -9580,14 +9580,14 @@
         <v>2.1871393585115584E-14</v>
       </c>
       <c r="E6">
-        <v>3.6509580173801999E-3</v>
+        <v>3.6509580173801201E-3</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>4.1078251911130792E-14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.9317880628477724E-14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>-5.5</v>
       </c>
@@ -9602,14 +9602,14 @@
         <v>1.1435297153639112E-13</v>
       </c>
       <c r="E7">
-        <v>4.02959998104726E-3</v>
+        <v>4.0295999810472504E-3</v>
       </c>
       <c r="F7">
         <f t="shared" si="1"/>
-        <v>1.9118040484045196E-13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.8873791418627661E-13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>-5.4</v>
       </c>
@@ -9624,14 +9624,14 @@
         <v>1.5765166949677223E-14</v>
       </c>
       <c r="E8">
-        <v>4.4469117443398497E-3</v>
+        <v>4.44691174433975E-3</v>
       </c>
       <c r="F8">
         <f t="shared" si="1"/>
-        <v>8.8817841970012523E-15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.3433698597964394E-14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>-5.3</v>
       </c>
@@ -9646,14 +9646,14 @@
         <v>1.8751666885918894E-13</v>
       </c>
       <c r="E9">
-        <v>4.9067147152196903E-3</v>
+        <v>4.9067147152197302E-3</v>
       </c>
       <c r="F9">
         <f t="shared" si="1"/>
-        <v>1.7108536809473662E-13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.6298074001497298E-13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>-5.2</v>
       </c>
@@ -9668,14 +9668,14 @@
         <v>5.5511151231257827E-15</v>
       </c>
       <c r="E10">
-        <v>5.4131810492571101E-3</v>
+        <v>5.4131810492570103E-3</v>
       </c>
       <c r="F10">
         <f t="shared" si="1"/>
-        <v>2.9531932455029164E-14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.1324274851176597E-14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>-5.0999999999999899</v>
       </c>
@@ -9690,14 +9690,14 @@
         <v>2.0206059048177849E-14</v>
       </c>
       <c r="E11">
-        <v>5.97086026487438E-3</v>
+        <v>5.9708602648744198E-3</v>
       </c>
       <c r="F11">
         <f t="shared" si="1"/>
-        <v>5.5289106626332796E-14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>6.1950444774083735E-14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>-5</v>
       </c>
@@ -9712,14 +9712,14 @@
         <v>1.5099033134902129E-14</v>
       </c>
       <c r="E12">
-        <v>6.5847067192883199E-3</v>
+        <v>6.5847067192882601E-3</v>
       </c>
       <c r="F12">
         <f t="shared" si="1"/>
-        <v>6.3726801613483985E-14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>5.4622972811557702E-14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>-4.9000000000000004</v>
       </c>
@@ -9734,14 +9734,14 @@
         <v>5.1070259132757201E-14</v>
       </c>
       <c r="E13">
-        <v>7.2601077096558098E-3</v>
+        <v>7.26010770965592E-3</v>
       </c>
       <c r="F13">
         <f t="shared" si="1"/>
-        <v>5.5511151231257827E-15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>9.7699626167013776E-15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>-4.8</v>
       </c>
@@ -9756,14 +9756,14 @@
         <v>4.75175454539567E-14</v>
       </c>
       <c r="E14">
-        <v>8.0029118968621398E-3</v>
+        <v>8.0029118968620895E-3</v>
       </c>
       <c r="F14">
         <f t="shared" si="1"/>
-        <v>3.7525538232330291E-14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4.3742787170231168E-14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>-4.7</v>
       </c>
@@ -9778,14 +9778,14 @@
         <v>1.5765166949677223E-14</v>
       </c>
       <c r="E15">
-        <v>8.8194576736365105E-3</v>
+        <v>8.8194576736365504E-3</v>
       </c>
       <c r="F15">
         <f t="shared" si="1"/>
-        <v>3.6193270602780103E-14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>3.1641356201816961E-14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>-4.5999999999999996</v>
       </c>
@@ -9800,14 +9800,14 @@
         <v>4.4297898682543746E-14</v>
       </c>
       <c r="E16">
-        <v>9.7166010148825796E-3</v>
+        <v>9.7166010148826004E-3</v>
       </c>
       <c r="F16">
         <f t="shared" si="1"/>
-        <v>2.7866597918091429E-14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.5757174171303632E-14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>-4.5</v>
       </c>
@@ -9829,7 +9829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>-4.4000000000000004</v>
       </c>
@@ -9851,7 +9851,7 @@
         <v>8.5487172896137054E-15</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>-4.3</v>
       </c>
@@ -9866,14 +9866,14 @@
         <v>6.9499961341534799E-14</v>
       </c>
       <c r="E19">
-        <v>1.2968489488436E-2</v>
+        <v>1.2968489488435901E-2</v>
       </c>
       <c r="F19">
         <f t="shared" si="1"/>
-        <v>3.8413716652030416E-14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+        <v>3.0864200084579352E-14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>-4.2</v>
       </c>
@@ -9888,14 +9888,14 @@
         <v>2.0983215165415459E-14</v>
       </c>
       <c r="E20">
-        <v>1.42678303084341E-2</v>
+        <v>1.4267830308433999E-2</v>
       </c>
       <c r="F20">
         <f t="shared" si="1"/>
-        <v>7.1054273576010019E-15</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.4099832412739488E-14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>-4.0999999999999996</v>
       </c>
@@ -9917,7 +9917,7 @@
         <v>6.4392935428259079E-15</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>-4</v>
       </c>
@@ -9932,14 +9932,14 @@
         <v>3.4861002973229915E-14</v>
       </c>
       <c r="E22">
-        <v>1.7247453008179099E-2</v>
+        <v>1.72474530081792E-2</v>
       </c>
       <c r="F22">
         <f t="shared" si="1"/>
-        <v>1.1546319456101628E-14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.7319479184152442E-14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>-3.9</v>
       </c>
@@ -9954,14 +9954,14 @@
         <v>0</v>
       </c>
       <c r="E23">
-        <v>1.89492452914552E-2</v>
+        <v>1.8949245291455301E-2</v>
       </c>
       <c r="F23">
         <f t="shared" si="1"/>
-        <v>7.9047879353311146E-14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7.382983113757291E-14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>-3.8</v>
       </c>
@@ -9983,7 +9983,7 @@
         <v>4.8849813083506888E-15</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>-3.7</v>
       </c>
@@ -9998,14 +9998,14 @@
         <v>1.3566925360919413E-13</v>
       </c>
       <c r="E25">
-        <v>2.2835331135848201E-2</v>
+        <v>2.2835331135848101E-2</v>
       </c>
       <c r="F25">
         <f t="shared" si="1"/>
-        <v>4.3742787170231168E-14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4.8183679268731794E-14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>-3.6</v>
       </c>
@@ -10020,14 +10020,14 @@
         <v>2.9154456626656611E-13</v>
       </c>
       <c r="E26">
-        <v>2.5044891848636699E-2</v>
+        <v>2.5044891848636799E-2</v>
       </c>
       <c r="F26">
         <f t="shared" si="1"/>
-        <v>3.1974423109204508E-14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.7977620220553945E-14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>-3.5</v>
       </c>
@@ -10049,7 +10049,7 @@
         <v>1.8207657603852567E-14</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>-3.4</v>
       </c>
@@ -10064,14 +10064,14 @@
         <v>1.0644818360106001E-12</v>
       </c>
       <c r="E28">
-        <v>3.0064513399361701E-2</v>
+        <v>3.0064513399361802E-2</v>
       </c>
       <c r="F28">
         <f t="shared" si="1"/>
-        <v>1.3322676295501878E-14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.6653345369377348E-14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>-3.3</v>
       </c>
@@ -10086,14 +10086,14 @@
         <v>1.5865087021893487E-12</v>
       </c>
       <c r="E29">
-        <v>3.2903092679469899E-2</v>
+        <v>3.2903092679470003E-2</v>
       </c>
       <c r="F29">
         <f t="shared" si="1"/>
-        <v>3.0420110874729289E-14</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+        <v>3.3528735343679728E-14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>-3.2</v>
       </c>
@@ -10108,14 +10108,14 @@
         <v>2.6458835122866731E-12</v>
       </c>
       <c r="E30">
-        <v>3.5980574260990002E-2</v>
+        <v>3.5980574260990099E-2</v>
       </c>
       <c r="F30">
         <f t="shared" si="1"/>
-        <v>5.5511151231257827E-15</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+        <v>8.2156503822261584E-15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>-3.1</v>
       </c>
@@ -10137,7 +10137,7 @@
         <v>7.5495165674510645E-15</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>-3</v>
       </c>
@@ -10159,7 +10159,7 @@
         <v>2.2204460492503131E-15</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>-2.9</v>
       </c>
@@ -10174,14 +10174,14 @@
         <v>1.2138956506646537E-11</v>
       </c>
       <c r="E33">
-        <v>4.6799574748099503E-2</v>
+        <v>4.6799574748099398E-2</v>
       </c>
       <c r="F33">
         <f t="shared" si="1"/>
-        <v>1.4988010832439613E-14</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.7208456881689926E-14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>-2.8</v>
       </c>
@@ -10196,14 +10196,14 @@
         <v>1.9640511439433794E-11</v>
       </c>
       <c r="E34">
-        <v>5.0986520273590602E-2</v>
+        <v>5.0986520273590498E-2</v>
       </c>
       <c r="F34">
         <f t="shared" si="1"/>
-        <v>1.5765166949677223E-14</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.3766765505351941E-14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>-2.7</v>
       </c>
@@ -10225,7 +10225,7 @@
         <v>8.992806499463768E-15</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>-2.6</v>
       </c>
@@ -10240,14 +10240,14 @@
         <v>4.8618886694384855E-11</v>
       </c>
       <c r="E36">
-        <v>6.0324097951421699E-2</v>
+        <v>6.0324097951421601E-2</v>
       </c>
       <c r="F36">
         <f t="shared" si="1"/>
-        <v>9.9920072216264089E-15</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.1657341758564144E-14</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>-2.4999999999999898</v>
       </c>
@@ -10262,14 +10262,14 @@
         <v>7.4342532130344807E-11</v>
       </c>
       <c r="E37">
-        <v>6.5504833187183503E-2</v>
+        <v>6.5504833187183406E-2</v>
       </c>
       <c r="F37">
         <f t="shared" si="1"/>
-        <v>2.4313884239290928E-14</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.5868196473766147E-14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>-2.4</v>
       </c>
@@ -10284,14 +10284,14 @@
         <v>1.0852230225566473E-10</v>
       </c>
       <c r="E38">
-        <v>7.1046205402122697E-2</v>
+        <v>7.1046205402122795E-2</v>
       </c>
       <c r="F38">
         <f t="shared" si="1"/>
-        <v>5.6621374255882984E-15</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4.3298697960381105E-15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>-2.2999999999999901</v>
       </c>
@@ -10306,14 +10306,14 @@
         <v>1.5680212683832906E-10</v>
       </c>
       <c r="E39">
-        <v>7.69619836702293E-2</v>
+        <v>7.6961983670229203E-2</v>
       </c>
       <c r="F39">
         <f t="shared" si="1"/>
-        <v>6.4392935428259079E-15</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7.7715611723760958E-15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>-2.2000000000000002</v>
       </c>
@@ -10328,14 +10328,14 @@
         <v>2.1931723104273715E-10</v>
       </c>
       <c r="E40">
-        <v>8.3265205232766995E-2</v>
+        <v>8.3265205232766898E-2</v>
       </c>
       <c r="F40">
         <f t="shared" si="1"/>
-        <v>2.3980817331903381E-14</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.5202062658991053E-14</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>-2.1</v>
       </c>
@@ -10350,14 +10350,14 @@
         <v>2.9487123853755293E-10</v>
       </c>
       <c r="E41">
-        <v>8.9968065889595897E-2</v>
+        <v>8.9968065889595994E-2</v>
       </c>
       <c r="F41">
         <f t="shared" si="1"/>
-        <v>1.4432899320127035E-14</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.532107773982716E-14</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>-1.99999999999999</v>
       </c>
@@ -10372,14 +10372,14 @@
         <v>3.7649994233390771E-10</v>
       </c>
       <c r="E42">
-        <v>9.7081821932948995E-2</v>
+        <v>9.7081821932948897E-2</v>
       </c>
       <c r="F42">
         <f t="shared" si="1"/>
-        <v>2.0650148258027912E-14</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.9539925233402755E-14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>-1.8999999999999899</v>
       </c>
@@ -10401,7 +10401,7 @@
         <v>4.7961634663806763E-14</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>-1.8</v>
       </c>
@@ -10423,7 +10423,7 @@
         <v>1.1546319456101628E-13</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>-1.7</v>
       </c>
@@ -10445,7 +10445,7 @@
         <v>2.3980817331903381E-13</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>-1.6</v>
       </c>
@@ -10467,7 +10467,7 @@
         <v>2.3869795029440866E-13</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>-1.5</v>
       </c>
@@ -10489,7 +10489,7 @@
         <v>4.0234482412415673E-13</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>-1.3999999999999899</v>
       </c>
@@ -10511,7 +10511,7 @@
         <v>8.0602191587786365E-13</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>-1.3</v>
       </c>
@@ -10533,7 +10533,7 @@
         <v>1.6404655411861313E-12</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>-1.2</v>
       </c>
@@ -10555,7 +10555,7 @@
         <v>3.2573943542502093E-12</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>-1.0999999999999901</v>
       </c>
@@ -10577,7 +10577,7 @@
         <v>6.3677951800400479E-12</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>-1</v>
       </c>
@@ -10599,7 +10599,7 @@
         <v>2.8565816379000353E-11</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>-0.89999999999999902</v>
       </c>
@@ -10621,7 +10621,7 @@
         <v>4.8841375388519737E-11</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>-0.8</v>
       </c>
@@ -10636,14 +10636,14 @@
         <v>5.0345712043764479E-8</v>
       </c>
       <c r="E54">
-        <v>0.21707540891139199</v>
+        <v>0.21707540891139099</v>
       </c>
       <c r="F54">
         <f t="shared" si="1"/>
-        <v>7.2251316041160862E-11</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+        <v>7.2246653104457437E-11</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>-0.7</v>
       </c>
@@ -10665,7 +10665,7 @@
         <v>1.1031686675266883E-10</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>-0.59999999999999898</v>
       </c>
@@ -10687,7 +10687,7 @@
         <v>1.5967915878434269E-10</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>-0.5</v>
       </c>
@@ -10709,7 +10709,7 @@
         <v>2.1678658868040657E-10</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>-0.39999999999999902</v>
       </c>
@@ -10724,14 +10724,14 @@
         <v>1.6923187751149982E-7</v>
       </c>
       <c r="E58">
-        <v>0.27165529744903999</v>
+        <v>0.27165529744903899</v>
       </c>
       <c r="F58">
         <f t="shared" si="1"/>
-        <v>2.7060376162069133E-10</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2.7060020890701253E-10</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>-0.3</v>
       </c>
@@ -10753,7 +10753,7 @@
         <v>2.9727109662758266E-10</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>-0.19999999999999901</v>
       </c>
@@ -10775,7 +10775,7 @@
         <v>2.5259705438429592E-10</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>-9.9999999999999797E-2</v>
       </c>
@@ -10790,14 +10790,14 @@
         <v>3.7892705007092076E-7</v>
       </c>
       <c r="E61">
-        <v>0.31720806675537699</v>
+        <v>0.31720806675537799</v>
       </c>
       <c r="F61">
         <f t="shared" si="1"/>
-        <v>6.3737237709915462E-11</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+        <v>6.3740568378989337E-11</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" s="1">
         <v>-2.2204460492503101E-16</v>
       </c>
@@ -10819,8 +10819,9 @@
         <v>3.8204883701098424E-10</v>
       </c>
       <c r="H62" s="1"/>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I62" s="1"/>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>9.9999999999999603E-2</v>
       </c>
@@ -10835,14 +10836,14 @@
         <v>5.2412538131818565E-7</v>
       </c>
       <c r="E63">
-        <v>0.34969263903887099</v>
+        <v>0.34969263903887199</v>
       </c>
       <c r="F63">
         <f t="shared" si="1"/>
-        <v>1.2580219088675904E-9</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.2580190222877263E-9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>0.19999999999999901</v>
       </c>
@@ -10864,7 +10865,7 @@
         <v>2.7802863344916773E-9</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>0.3</v>
       </c>
@@ -10886,7 +10887,7 @@
         <v>5.2444035780752074E-9</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>0.4</v>
       </c>
@@ -10908,7 +10909,7 @@
         <v>5.6115494473374383E-9</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>0.5</v>
       </c>
@@ -10930,7 +10931,7 @@
         <v>9.8889976207772179E-9</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>0.59999999999999898</v>
       </c>
@@ -10952,7 +10953,7 @@
         <v>1.6079777287458796E-8</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>0.69999999999999896</v>
       </c>
@@ -10974,7 +10975,7 @@
         <v>2.4592849423576979E-8</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>0.8</v>
       </c>
@@ -10989,14 +10990,14 @@
         <v>1.0242802384041738E-6</v>
       </c>
       <c r="E70">
-        <v>0.47598642097918198</v>
+        <v>0.47598642097918098</v>
       </c>
       <c r="F70">
         <f t="shared" si="3"/>
-        <v>3.5383043939241077E-8</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+        <v>3.5383046048664824E-8</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>0.89999999999999902</v>
       </c>
@@ -11018,7 +11019,7 @@
         <v>4.9790182310438524E-8</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>0.999999999999999</v>
       </c>
@@ -11040,7 +11041,7 @@
         <v>1.1105112307507881E-7</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>1.0999999999999901</v>
       </c>
@@ -11062,7 +11063,7 @@
         <v>1.0357972823893391E-7</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>1.19999999999999</v>
       </c>
@@ -11084,7 +11085,7 @@
         <v>1.2667446613878752E-7</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>1.3</v>
       </c>
@@ -11106,7 +11107,7 @@
         <v>1.4671351722395087E-7</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>1.3999999999999899</v>
       </c>
@@ -11128,7 +11129,7 @@
         <v>1.6499544319703574E-7</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>1.5</v>
       </c>
@@ -11150,7 +11151,7 @@
         <v>2.2338193295112774E-7</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>1.6</v>
       </c>
@@ -11172,7 +11173,7 @@
         <v>2.3250991654233388E-7</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>1.7</v>
       </c>
@@ -11194,7 +11195,7 @@
         <v>3.1275613654457857E-8</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>1.8</v>
       </c>
@@ -11209,14 +11210,14 @@
         <v>3.2972335594294577E-5</v>
       </c>
       <c r="E80">
-        <v>0.68859507527249397</v>
+        <v>0.68859507527249297</v>
       </c>
       <c r="F80">
         <f t="shared" si="3"/>
-        <v>1.6161475580034335E-7</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.6161475446807572E-7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>1.9</v>
       </c>
@@ -11238,7 +11239,7 @@
         <v>3.149945406732968E-7</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>1.99999999999999</v>
       </c>
@@ -11260,7 +11261,7 @@
         <v>6.000734524835849E-7</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>2.1</v>
       </c>
@@ -11275,14 +11276,14 @@
         <v>5.1047389395542098E-5</v>
       </c>
       <c r="E83">
-        <v>0.76030670818393498</v>
+        <v>0.76030670818394197</v>
       </c>
       <c r="F83">
         <f t="shared" si="3"/>
-        <v>1.0019068330535674E-6</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.0019068421573962E-6</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>2.2000000000000002</v>
       </c>
@@ -11297,14 +11298,14 @@
         <v>5.5954774599076273E-5</v>
       </c>
       <c r="E84">
-        <v>0.78526387394128305</v>
+        <v>0.78526387394129105</v>
       </c>
       <c r="F84">
         <f t="shared" si="3"/>
-        <v>1.9248254703452261E-6</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.9248254805592779E-6</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>2.2999999999999998</v>
       </c>
@@ -11319,14 +11320,14 @@
         <v>5.7665584450194984E-5</v>
       </c>
       <c r="E85">
-        <v>0.81089831189682005</v>
+        <v>0.81089831189682804</v>
       </c>
       <c r="F85">
         <f t="shared" si="3"/>
-        <v>2.1904909046632781E-6</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.1904909146552853E-6</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>2.3999999999999901</v>
       </c>
@@ -11341,14 +11342,14 @@
         <v>4.8857028744464515E-5</v>
       </c>
       <c r="E86">
-        <v>0.83748782513982101</v>
+        <v>0.837487825139829</v>
       </c>
       <c r="F86">
         <f t="shared" si="3"/>
-        <v>2.2010848779174808E-6</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.2010848874653988E-6</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>2.4999999999999898</v>
       </c>
@@ -11363,14 +11364,14 @@
         <v>2.6762659625090279E-5</v>
       </c>
       <c r="E87">
-        <v>0.86597658169341896</v>
+        <v>0.86597658169253999</v>
       </c>
       <c r="F87">
         <f t="shared" si="3"/>
-        <v>2.6814328810687016E-6</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.6814318661028125E-6</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>2.6</v>
       </c>
@@ -11385,14 +11386,14 @@
         <v>1.4094537626796466E-5</v>
       </c>
       <c r="E88">
-        <v>0.89545158993409302</v>
+        <v>0.89545158993302798</v>
       </c>
       <c r="F88">
         <f t="shared" si="3"/>
-        <v>2.6305790117309158E-6</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.6305778222379672E-6</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>2.7</v>
       </c>
@@ -11407,14 +11408,14 @@
         <v>1.1143721897033387E-5</v>
       </c>
       <c r="E89">
-        <v>0.92552692470490106</v>
+        <v>0.92552692450561702</v>
       </c>
       <c r="F89">
         <f t="shared" si="3"/>
-        <v>2.3824640933423069E-6</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.3822487731361974E-6</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>2.8</v>
       </c>
@@ -11429,14 +11430,14 @@
         <v>8.7959817480776081E-6</v>
       </c>
       <c r="E90">
-        <v>0.95605485900509801</v>
+        <v>0.95605485903654397</v>
       </c>
       <c r="F90">
         <f t="shared" si="3"/>
-        <v>2.0172683945496317E-6</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.0173012860169592E-6</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>2.9</v>
       </c>
@@ -11451,14 +11452,14 @@
         <v>6.8818506964163362E-6</v>
       </c>
       <c r="E91">
-        <v>0.98694542538483598</v>
+        <v>0.98694542613424296</v>
       </c>
       <c r="F91">
         <f t="shared" si="3"/>
-        <v>1.6596062042406601E-6</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.6603655250690963E-6</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>3</v>
       </c>
@@ -11473,14 +11474,14 @@
         <v>5.5286297750978264E-6</v>
       </c>
       <c r="E92">
-        <v>1.01813601805843</v>
+        <v>1.01813601805812</v>
       </c>
       <c r="F92">
         <f t="shared" si="3"/>
-        <v>1.4557962801919899E-6</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.4557959757688366E-6</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>3.1</v>
       </c>
@@ -11495,14 +11496,14 @@
         <v>4.4216355914450389E-6</v>
       </c>
       <c r="E93">
-        <v>1.0495829007314501</v>
+        <v>1.0495795282249301</v>
       </c>
       <c r="F93">
         <f t="shared" si="3"/>
-        <v>4.4216355914450389E-6</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.2084340144102867E-6</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>3.2</v>
       </c>
@@ -11517,14 +11518,14 @@
         <v>3.548506897210757E-6</v>
       </c>
       <c r="E94">
-        <v>1.08123937067534</v>
+        <v>1.0812393715804101</v>
       </c>
       <c r="F94">
         <f t="shared" si="3"/>
-        <v>9.7852029257161632E-7</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+        <v>9.793573605421102E-7</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>3.3</v>
       </c>
@@ -11539,14 +11540,14 @@
         <v>2.7985853503498248E-6</v>
       </c>
       <c r="E95">
-        <v>1.11308606946918</v>
+        <v>1.11308606945438</v>
       </c>
       <c r="F95">
         <f t="shared" si="3"/>
-        <v>7.7933714193179071E-7</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7.793238456788032E-7</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>3.4</v>
       </c>
@@ -11561,14 +11562,14 @@
         <v>2.2181361067907801E-6</v>
       </c>
       <c r="E96">
-        <v>1.14509537409171</v>
+        <v>1.1450953733087801</v>
       </c>
       <c r="F96">
         <f t="shared" si="3"/>
-        <v>6.0827867232049471E-7</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+        <v>6.0759494724393903E-7</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>3.5</v>
       </c>
@@ -11583,14 +11584,14 @@
         <v>1.7641660650102864E-6</v>
       </c>
       <c r="E97">
-        <v>1.1772470231448899</v>
+        <v>1.1772470231515</v>
       </c>
       <c r="F97">
         <f t="shared" si="3"/>
-        <v>4.6622668414819657E-7</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4.6623229899012131E-7</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>3.6</v>
       </c>
@@ -11605,14 +11606,14 @@
         <v>1.3997863690384804E-6</v>
       </c>
       <c r="E98">
-        <v>1.20952513706467</v>
+        <v>1.20952386781355</v>
       </c>
       <c r="F98">
         <f t="shared" si="3"/>
-        <v>1.3997863690384804E-6</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+        <v>3.504052046299222E-7</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>3.7</v>
       </c>
@@ -11627,14 +11628,14 @@
         <v>1.1089460489888125E-6</v>
       </c>
       <c r="E99">
-        <v>1.2419123081180301</v>
+        <v>1.24191125239753</v>
       </c>
       <c r="F99">
         <f t="shared" si="3"/>
-        <v>1.1089460489888125E-6</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.5886858057155848E-7</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>3.8</v>
       </c>
@@ -11649,14 +11650,14 @@
         <v>8.7783116820006057E-7</v>
       </c>
       <c r="E100">
-        <v>1.2743965507557999</v>
+        <v>1.2743965507797801</v>
       </c>
       <c r="F100">
         <f t="shared" si="3"/>
-        <v>1.9035024534375111E-7</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.9036906206970627E-7</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>3.9</v>
       </c>
@@ -11671,14 +11672,14 @@
         <v>6.9484619813486859E-7</v>
       </c>
       <c r="E101">
-        <v>1.3069688079544599</v>
+        <v>1.3069688079605599</v>
       </c>
       <c r="F101">
         <f t="shared" si="3"/>
-        <v>1.4015218607887903E-7</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.4015685345647455E-7</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>4</v>
       </c>
@@ -11693,14 +11694,14 @@
         <v>5.5025899037275394E-7</v>
       </c>
       <c r="E102">
-        <v>1.33961846754282</v>
+        <v>1.3396184676107401</v>
       </c>
       <c r="F102">
         <f t="shared" si="3"/>
-        <v>1.0215985923878179E-7</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.0221056023773656E-7</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>4.0999999999999996</v>
       </c>
@@ -11715,14 +11716,14 @@
         <v>4.3612693101380273E-7</v>
       </c>
       <c r="E103">
-        <v>1.3723371457990601</v>
+        <v>1.37233716032428</v>
       </c>
       <c r="F103">
         <f t="shared" si="3"/>
-        <v>6.329168145136066E-8</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7.3875976225323825E-8</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>4.2</v>
       </c>
@@ -11737,14 +11738,14 @@
         <v>3.4607692755983521E-7</v>
       </c>
       <c r="E104">
-        <v>1.4051175110440299</v>
+        <v>1.4051175246605301</v>
       </c>
       <c r="F104">
         <f t="shared" si="3"/>
-        <v>4.3287819107007408E-8</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+        <v>5.2978468056963379E-8</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>4.3</v>
       </c>
@@ -11759,14 +11760,14 @@
         <v>2.7490233489579907E-7</v>
       </c>
       <c r="E105">
-        <v>1.4379530632627699</v>
+        <v>1.437953059656</v>
       </c>
       <c r="F105">
         <f t="shared" si="3"/>
-        <v>3.7269541897089198E-8</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+        <v>3.4761274969596911E-8</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>4.4000000000000004</v>
       </c>
@@ -11781,14 +11782,14 @@
         <v>2.1866385191415816E-7</v>
       </c>
       <c r="E106">
-        <v>1.4708380278836399</v>
+        <v>1.47083802714492</v>
       </c>
       <c r="F106">
         <f t="shared" si="3"/>
-        <v>2.6611679970756086E-8</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.6109435724563923E-8</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>4.5</v>
       </c>
@@ -11803,14 +11804,14 @@
         <v>1.7414171882279561E-7</v>
       </c>
       <c r="E107">
-        <v>1.5037673139049299</v>
+        <v>1.5037673145508099</v>
       </c>
       <c r="F107">
         <f t="shared" si="3"/>
-        <v>1.8128855527876908E-8</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.8558363512610754E-8</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>4.5999999999999996</v>
       </c>
@@ -11825,14 +11826,14 @@
         <v>1.3884142702202951E-7</v>
       </c>
       <c r="E108">
-        <v>1.5367365808270601</v>
+        <v>1.53673638683071</v>
       </c>
       <c r="F108">
         <f t="shared" si="3"/>
-        <v>1.3884142702202951E-7</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.2602239696235529E-8</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>4.7</v>
       </c>
@@ -11847,14 +11848,14 @@
         <v>1.108072853472919E-7</v>
       </c>
       <c r="E109">
-        <v>1.5697412039142</v>
+        <v>1.5697412038579801</v>
       </c>
       <c r="F109">
         <f t="shared" si="3"/>
-        <v>8.918725091788815E-9</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+        <v>8.8829101851928272E-9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>4.8</v>
       </c>
@@ -11869,14 +11870,14 @@
         <v>8.8508587570146346E-8</v>
       </c>
       <c r="E110">
-        <v>1.6027781558760299</v>
+        <v>1.6027781569606401</v>
       </c>
       <c r="F110">
         <f t="shared" si="3"/>
-        <v>5.3184776582781979E-9</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+        <v>5.9951841269167971E-9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>4.9000000000000004</v>
       </c>
@@ -11891,14 +11892,14 @@
         <v>7.0742441682369872E-8</v>
       </c>
       <c r="E111">
-        <v>1.6358440227945801</v>
+        <v>1.6358440090701201</v>
       </c>
       <c r="F111">
         <f t="shared" si="3"/>
-        <v>3.9748777602710561E-9</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4.4149564004669628E-9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>5</v>
       </c>
@@ -11913,14 +11914,14 @@
         <v>5.6572064588422677E-8</v>
       </c>
       <c r="E112">
-        <v>1.6689359155358801</v>
+        <v>1.6689359162963799</v>
       </c>
       <c r="F112">
         <f t="shared" si="3"/>
-        <v>2.147691802178997E-9</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.6033712963169364E-9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>5.0999999999999996</v>
       </c>
@@ -11935,14 +11936,14 @@
         <v>4.5254295200081174E-8</v>
       </c>
       <c r="E113">
-        <v>1.7020512518270501</v>
+        <v>1.7020512395446601</v>
       </c>
       <c r="F113">
         <f t="shared" si="3"/>
-        <v>1.2598797560769981E-9</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+        <v>5.9563483034708042E-9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>5.2</v>
       </c>
@@ -11957,14 +11958,14 @@
         <v>3.6197265407267309E-8</v>
       </c>
       <c r="E114">
-        <v>1.73518771318884</v>
+        <v>1.7351877123452699</v>
       </c>
       <c r="F114">
         <f t="shared" si="3"/>
-        <v>1.0405907246990864E-9</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+        <v>5.5443560853518647E-10</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>5.3</v>
       </c>
@@ -11979,14 +11980,14 @@
         <v>2.8937487739355561E-8</v>
       </c>
       <c r="E115">
-        <v>1.7683432672897399</v>
+        <v>1.7683432162069399</v>
       </c>
       <c r="F115">
         <f t="shared" si="3"/>
-        <v>2.8937487739355561E-8</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+        <v>5.010902803803674E-11</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>5.4</v>
       </c>
@@ -12001,14 +12002,14 @@
         <v>2.3081128563973152E-8</v>
       </c>
       <c r="E116">
-        <v>1.8015158949419301</v>
+        <v>1.80151589084748</v>
       </c>
       <c r="F116">
         <f t="shared" si="3"/>
-        <v>3.3152636191857709E-10</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.9412540464003314E-9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>5.5</v>
       </c>
@@ -12023,14 +12024,14 @@
         <v>1.3349542582474783E-8</v>
       </c>
       <c r="E117">
-        <v>1.83470406450707</v>
+        <v>1.8347040652569899</v>
       </c>
       <c r="F117">
         <f t="shared" si="3"/>
-        <v>3.9087499903445178E-10</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.7866597090687719E-11</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>5.6</v>
       </c>
@@ -12045,14 +12046,14 @@
         <v>1.0493123037136343E-8</v>
       </c>
       <c r="E118">
-        <v>1.8679062166874001</v>
+        <v>1.86790621666811</v>
       </c>
       <c r="F118">
         <f t="shared" si="3"/>
-        <v>4.5296655315496537E-11</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+        <v>3.4969582785038256E-11</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>5.7</v>
       </c>
@@ -12067,14 +12068,14 @@
         <v>8.2485280827881979E-9</v>
       </c>
       <c r="E119">
-        <v>1.90112098269354</v>
+        <v>1.9011209872622801</v>
       </c>
       <c r="F119">
         <f t="shared" si="3"/>
-        <v>2.421587153023097E-9</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1.8404944235328458E-11</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>5.8</v>
       </c>
@@ -12089,14 +12090,14 @@
         <v>6.4843117542068285E-9</v>
       </c>
       <c r="E120">
-        <v>1.9343471512897099</v>
+        <v>1.93434715121235</v>
       </c>
       <c r="F120">
         <f t="shared" si="3"/>
-        <v>5.197098307263559E-11</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+        <v>9.1963769932590367E-11</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>5.9</v>
       </c>
@@ -12111,14 +12112,14 @@
         <v>5.0994986011687615E-9</v>
       </c>
       <c r="E121">
-        <v>1.9675836040880801</v>
+        <v>1.9675835999989699</v>
       </c>
       <c r="F121">
         <f t="shared" si="3"/>
-        <v>9.6163632612444871E-11</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.174403213039966E-9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>6</v>
       </c>
@@ -12133,11 +12134,11 @@
         <v>4.0107419607693373E-9</v>
       </c>
       <c r="E122">
-        <v>2.0008293501173502</v>
+        <v>2.0008293501172898</v>
       </c>
       <c r="F122">
         <f t="shared" si="3"/>
-        <v>6.5787597591793201E-11</v>
+        <v>6.5817795658063005E-11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>